<commit_message>
Update best-known values and benchmark summary
</commit_message>
<xml_diff>
--- a/summary_results.xlsx
+++ b/summary_results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thanh Tu\Downloads\FCBQP_parallel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\users\thanh tu\Downloads\FCBQP_parallel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E4C2D0-54DE-4549-9E98-4E34EFD908A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9B5A37-87C1-4026-81B6-9EDBDBB2B6C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{82BDEFC4-01A7-4C40-9695-256D581AEFD9}"/>
   </bookViews>
@@ -9073,7 +9073,7 @@
         <v>3.24225E-2</v>
       </c>
       <c r="F129">
-        <v>19725322.192839898</v>
+        <v>19725322.192839999</v>
       </c>
       <c r="G129">
         <v>19725322.192839999</v>
@@ -9129,7 +9129,7 @@
         <v>3.24225E-2</v>
       </c>
       <c r="F130">
-        <v>23805405.245379899</v>
+        <v>23805405.245379999</v>
       </c>
       <c r="G130">
         <v>23805405.245379899</v>
@@ -9297,7 +9297,7 @@
         <v>3.1032219999999999E-2</v>
       </c>
       <c r="F133">
-        <v>21260902.726679899</v>
+        <v>21260902.726679999</v>
       </c>
       <c r="G133">
         <v>21260902.726679999</v>
@@ -9353,7 +9353,7 @@
         <v>3.1032219999999999E-2</v>
       </c>
       <c r="F134">
-        <v>30495483.292709898</v>
+        <v>30495483.292709999</v>
       </c>
       <c r="G134">
         <v>30495483.292709898</v>
@@ -9409,7 +9409,7 @@
         <v>3.1032219999999999E-2</v>
       </c>
       <c r="F135">
-        <v>38032901.950429901</v>
+        <v>38032901.950429998</v>
       </c>
       <c r="G135">
         <v>38032901.950429797</v>
@@ -9577,7 +9577,7 @@
         <v>2.930408E-2</v>
       </c>
       <c r="F138">
-        <v>22840863.487539899</v>
+        <v>22840863.487539999</v>
       </c>
       <c r="G138">
         <v>22840863.487539999</v>
@@ -9689,7 +9689,7 @@
         <v>2.930408E-2</v>
       </c>
       <c r="F140">
-        <v>55943547.515639901</v>
+        <v>55943547.515639998</v>
       </c>
       <c r="G140">
         <v>55943547.515639998</v>
@@ -9857,7 +9857,7 @@
         <v>3.1367609999999997E-2</v>
       </c>
       <c r="F143">
-        <v>23074932.414009899</v>
+        <v>23074932.414009999</v>
       </c>
       <c r="G143">
         <v>23074932.414009999</v>
@@ -9913,7 +9913,7 @@
         <v>3.1367609999999997E-2</v>
       </c>
       <c r="F144">
-        <v>40469681.9321099</v>
+        <v>40469681.932109997</v>
       </c>
       <c r="G144">
         <v>40469681.932109997</v>
@@ -9969,7 +9969,7 @@
         <v>3.1367609999999997E-2</v>
       </c>
       <c r="F145">
-        <v>62332519.3934699</v>
+        <v>62332519.393469997</v>
       </c>
       <c r="G145">
         <v>62332519.3934699</v>
@@ -12486,7 +12486,7 @@
         <v>0.99950000000000006</v>
       </c>
       <c r="F190">
-        <v>11292398.161482001</v>
+        <v>11292398.161481</v>
       </c>
       <c r="G190">
         <v>11292398.1614813</v>
@@ -12542,7 +12542,7 @@
         <v>0.99950000000000006</v>
       </c>
       <c r="F191">
-        <v>11299940.462685</v>
+        <v>11299940.462684</v>
       </c>
       <c r="G191">
         <v>11299940.4626841</v>
@@ -12598,7 +12598,7 @@
         <v>0.99950000000000006</v>
       </c>
       <c r="F192">
-        <v>11291119.490684001</v>
+        <v>11291119.490683001</v>
       </c>
       <c r="G192">
         <v>11291119.490683099</v>
@@ -12710,7 +12710,7 @@
         <v>0.99950000000000006</v>
       </c>
       <c r="F194">
-        <v>11298430.416818</v>
+        <v>11298430.416817</v>
       </c>
       <c r="G194">
         <v>11298430.416817401</v>
@@ -12766,7 +12766,7 @@
         <v>0.99950000000000006</v>
       </c>
       <c r="F195">
-        <v>11305676.848937901</v>
+        <v>11305676.848937999</v>
       </c>
       <c r="G195">
         <v>11305676.8489378</v>
@@ -12822,7 +12822,7 @@
         <v>0.99950000000000006</v>
       </c>
       <c r="F196">
-        <v>11282910.8806899</v>
+        <v>11282910.880689999</v>
       </c>
       <c r="G196">
         <v>11282909.8929267</v>
@@ -13270,7 +13270,7 @@
         <v>0.99950000000000006</v>
       </c>
       <c r="F204">
-        <v>11302892.010384001</v>
+        <v>11302892.010383001</v>
       </c>
       <c r="G204">
         <v>11302892.010383099</v>
@@ -13546,11 +13546,11 @@
       <c r="F209" s="8"/>
       <c r="G209" s="8">
         <f t="array" ref="G209">AVERAGE((F189:F208-G189:G208)/F189:F208)</f>
-        <v>8.512985407919487E-6</v>
+        <v>8.512985386658379E-6</v>
       </c>
       <c r="H209" s="8">
         <f t="array" ref="H209">AVERAGE((F189:F208-H189:H208)/F189:F208)</f>
-        <v>6.8271909033567669E-5</v>
+        <v>6.8271909012309473E-5</v>
       </c>
       <c r="I209" s="8" t="s">
         <v>9</v>
@@ -13577,7 +13577,7 @@
       </c>
       <c r="P209" s="10">
         <f t="array" ref="P209">AVERAGE((F189:F208-P189:P208)/F189:F208)</f>
-        <v>3.757193501832543E-6</v>
+        <v>3.7571934805714866E-6</v>
       </c>
       <c r="Q209" s="8" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Update corrected SyntheticTF instances
</commit_message>
<xml_diff>
--- a/summary_results.xlsx
+++ b/summary_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thanh Tu\Downloads\FCBQP_parallel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29972222-0232-498A-B496-443C283EBE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2756553-02F2-4571-8F86-F65F752D3D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9540" windowWidth="29040" windowHeight="15720" xr2:uid="{82BDEFC4-01A7-4C40-9695-256D581AEFD9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{82BDEFC4-01A7-4C40-9695-256D581AEFD9}"/>
   </bookViews>
   <sheets>
     <sheet name="FCBQP_1core_5runs_summary" sheetId="1" r:id="rId1"/>
@@ -1214,13 +1214,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
-    <numFmt numFmtId="168" formatCode="0.0000000"/>
-    <numFmt numFmtId="169" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -1729,7 +1727,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1742,8 +1740,7 @@
     <xf numFmtId="10" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="169" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1753,6 +1750,10 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2113,6 +2114,7 @@
   <cols>
     <col min="1" max="1" width="29.44140625" customWidth="1"/>
     <col min="2" max="2" width="27.5546875" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" customWidth="1"/>
     <col min="6" max="6" width="24.33203125" customWidth="1"/>
     <col min="7" max="7" width="13.6640625" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
@@ -2127,24 +2129,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="13" t="s">
         <v>331</v>
       </c>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="15" t="s">
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="14" t="s">
         <v>332</v>
       </c>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="16" t="s">
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="15" t="s">
         <v>333</v>
       </c>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
+      <c r="P1" s="15"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="15"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -10939,7 +10941,7 @@
         <f t="array" ref="G160">AVERAGE((F150:F159-G150:G159)/F150:F159)</f>
         <v>4.8344748254018773E-5</v>
       </c>
-      <c r="H160" s="8">
+      <c r="H160" s="12">
         <f t="array" ref="H160">AVERAGE((F150:F159-H150:H159)/F150:F159)</f>
         <v>2.3037513103146826E-4</v>
       </c>
@@ -10961,7 +10963,7 @@
         <f>SUM(N150:N159)</f>
         <v>45</v>
       </c>
-      <c r="O160" s="13">
+      <c r="O160" s="12">
         <f t="array" ref="O160">AVERAGE((F150:F159-O150:O159)/F150:F159)</f>
         <v>1.4982421786531849E-5</v>
       </c>
@@ -12106,11 +12108,11 @@
       <c r="D181" s="8"/>
       <c r="E181" s="9"/>
       <c r="F181" s="8"/>
-      <c r="G181" s="8">
+      <c r="G181" s="12">
         <f t="array" ref="G181">AVERAGE((F161:F180-G161:G180)/F161:F180)</f>
         <v>2.8800199951982885E-4</v>
       </c>
-      <c r="H181" s="8">
+      <c r="H181" s="12">
         <f t="array" ref="H181">AVERAGE((F161:F180-H161:H180)/F161:F180)</f>
         <v>3.9132569547953012E-4</v>
       </c>
@@ -12119,11 +12121,11 @@
         <f>SUM(J161:J180)</f>
         <v>3</v>
       </c>
-      <c r="K181" s="8">
+      <c r="K181" s="12">
         <f t="array" ref="K181">AVERAGE((F161:F180-K161:K180)/F161:F180)</f>
         <v>1.8818171579320272E-4</v>
       </c>
-      <c r="L181" s="8">
+      <c r="L181" s="12">
         <f t="array" ref="L181">AVERAGE((F161:F180-L161:L180)/F161:F180)</f>
         <v>2.1204684058721482E-4</v>
       </c>
@@ -12132,11 +12134,11 @@
         <f>SUM(N161:N180)</f>
         <v>37</v>
       </c>
-      <c r="O181" s="10">
+      <c r="O181" s="12">
         <f t="array" ref="O181">AVERAGE((F161:F180-O161:O180)/F161:F180)</f>
         <v>2.0842144795972422E-4</v>
       </c>
-      <c r="P181" s="10">
+      <c r="P181" s="12">
         <f t="array" ref="P181">AVERAGE((F161:F180-P161:P180)/F161:F180)</f>
         <v>2.5666646118477539E-4</v>
       </c>
@@ -12747,7 +12749,7 @@
         <f t="array" ref="O192">AVERAGE((F182:F191-O182:O191)/F182:F191)</f>
         <v>5.3575608518604454E-6</v>
       </c>
-      <c r="P192" s="10">
+      <c r="P192" s="12">
         <f t="array" ref="P192">AVERAGE((F182:F191-P182:P191)/F182:F191)</f>
         <v>1.2033231401112437E-5</v>
       </c>
@@ -13052,7 +13054,7 @@
         <f t="array" ref="G198">AVERAGE((F193:F197-G193:G197)/F193:F197)</f>
         <v>0</v>
       </c>
-      <c r="H198" s="8">
+      <c r="H198" s="12">
         <f t="array" ref="H198">AVERAGE((F193:F197-H193:H197)/F193:F197)</f>
         <v>1.1745823146463784E-3</v>
       </c>
@@ -13078,7 +13080,7 @@
         <f t="array" ref="O198">AVERAGE((F193:F197-O193:O197)/F193:F197)</f>
         <v>0</v>
       </c>
-      <c r="P198" s="8">
+      <c r="P198" s="12">
         <f t="array" ref="P198">AVERAGE((F193:F197-P193:P197)/F193:F197)</f>
         <v>2.0986867296829051E-4</v>
       </c>
@@ -13383,7 +13385,7 @@
         <f t="array" ref="G204">AVERAGE((F199:F203-G199:G203)/F199:F203)</f>
         <v>8.2027307913297974E-5</v>
       </c>
-      <c r="H204" s="8">
+      <c r="H204" s="12">
         <f t="array" ref="H204">AVERAGE((F199:F203-H199:H203)/F199:F203)</f>
         <v>2.7641821301519539E-4</v>
       </c>
@@ -13405,11 +13407,11 @@
         <f>SUM(N199:N203)</f>
         <v>24</v>
       </c>
-      <c r="O204" s="10">
+      <c r="O204" s="12">
         <f t="array" ref="O204">AVERAGE((F199:F203-O199:O203)/F199:F203)</f>
         <v>2.4393602879305516E-3</v>
       </c>
-      <c r="P204" s="10">
+      <c r="P204" s="12">
         <f t="array" ref="P204">AVERAGE((F199:F203-P199:P203)/F199:F203)</f>
         <v>6.3154452435111395E-3</v>
       </c>
@@ -13606,10 +13608,10 @@
       <c r="F208">
         <v>854.72222999999997</v>
       </c>
-      <c r="G208">
+      <c r="G208" s="16">
         <v>852.25382999999999</v>
       </c>
-      <c r="H208">
+      <c r="H208" s="16">
         <v>851.04265799999996</v>
       </c>
       <c r="I208" t="s">
@@ -13621,8 +13623,8 @@
       <c r="K208">
         <v>854.34204</v>
       </c>
-      <c r="L208">
-        <v>853.870676</v>
+      <c r="L208" s="16">
+        <v>853.78969400000005</v>
       </c>
       <c r="M208" t="s">
         <v>367</v>
@@ -13630,10 +13632,10 @@
       <c r="N208">
         <v>0</v>
       </c>
-      <c r="O208" s="2">
+      <c r="O208" s="18">
         <v>724.39059999999995</v>
       </c>
-      <c r="P208" s="2">
+      <c r="P208" s="18">
         <v>698.27013399999998</v>
       </c>
       <c r="Q208" t="s">
@@ -13710,11 +13712,11 @@
       <c r="D210" s="8"/>
       <c r="E210" s="9"/>
       <c r="F210" s="8"/>
-      <c r="G210" s="8">
+      <c r="G210" s="12">
         <f t="array" ref="G210">AVERAGE((F205:F209-G205:G209)/F205:F209)</f>
         <v>1.5590576978140082E-3</v>
       </c>
-      <c r="H210" s="8">
+      <c r="H210" s="12">
         <f t="array" ref="H210">AVERAGE((F205:F209-H205:H209)/F205:F209)</f>
         <v>2.6283403189026962E-3</v>
       </c>
@@ -13723,24 +13725,24 @@
         <f>SUM(J205:J209)</f>
         <v>6</v>
       </c>
-      <c r="K210" s="8">
+      <c r="K210" s="12">
         <f t="array" ref="K210">AVERAGE((F205:F209-K205:K209)/F205:F209)</f>
         <v>5.621798468248122E-4</v>
       </c>
-      <c r="L210" s="8">
+      <c r="L210" s="12">
         <f t="array" ref="L210">AVERAGE((F205:F209-L205:L209)/F205:F209)</f>
-        <v>7.4278865537821977E-4</v>
+        <v>7.6173796947291673E-4</v>
       </c>
       <c r="M210" s="8"/>
       <c r="N210" s="8">
         <f>SUM(N205:N209)</f>
         <v>9</v>
       </c>
-      <c r="O210" s="10">
+      <c r="O210" s="12">
         <f t="array" ref="O210">AVERAGE((F205:F209-O205:O209)/F205:F209)</f>
         <v>0.15775863556590949</v>
       </c>
-      <c r="P210" s="10">
+      <c r="P210" s="12">
         <f t="array" ref="P210">AVERAGE((F205:F209-P205:P209)/F205:F209)</f>
         <v>0.22715926564001485</v>
       </c>
@@ -13755,7 +13757,7 @@
         <v>392</v>
       </c>
       <c r="B211" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C211">
         <v>7000</v>
@@ -13764,40 +13766,40 @@
         <v>100</v>
       </c>
       <c r="E211" s="1">
-        <v>1.53294E-3</v>
-      </c>
-      <c r="F211">
-        <v>142.71664999999999</v>
-      </c>
-      <c r="G211">
-        <v>142.50523000000001</v>
+        <v>1.5150999999999999E-3</v>
+      </c>
+      <c r="F211" s="7">
+        <v>142.13679999999999</v>
+      </c>
+      <c r="G211" s="7">
+        <v>142.13679999999999</v>
       </c>
       <c r="H211">
-        <v>142.06044</v>
-      </c>
-      <c r="I211" t="s">
-        <v>367</v>
+        <v>142.07524599999999</v>
+      </c>
+      <c r="I211">
+        <v>35.900492999999997</v>
       </c>
       <c r="J211">
-        <v>0</v>
-      </c>
-      <c r="K211">
-        <v>142.71664999999999</v>
-      </c>
-      <c r="L211">
-        <v>142.71664999999999</v>
+        <v>2</v>
+      </c>
+      <c r="K211" s="7">
+        <v>142.13679999999999</v>
+      </c>
+      <c r="L211" s="2">
+        <v>142.13679999999999</v>
       </c>
       <c r="M211">
-        <v>8.920871</v>
+        <v>1.886042</v>
       </c>
       <c r="N211">
         <v>5</v>
       </c>
       <c r="O211" s="2">
-        <v>113.59756</v>
+        <v>97.164249999999996</v>
       </c>
       <c r="P211" s="2">
-        <v>109.171176</v>
+        <v>92.234967999999995</v>
       </c>
       <c r="Q211" t="s">
         <v>367</v>
@@ -13811,7 +13813,7 @@
         <v>392</v>
       </c>
       <c r="B212" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C212">
         <v>7000</v>
@@ -13820,16 +13822,16 @@
         <v>200</v>
       </c>
       <c r="E212" s="1">
-        <v>1.53294E-3</v>
-      </c>
-      <c r="F212">
-        <v>255.61268999999999</v>
-      </c>
-      <c r="G212">
-        <v>254.78677999999999</v>
+        <v>1.5150999999999999E-3</v>
+      </c>
+      <c r="F212" s="7">
+        <v>247.79705999999999</v>
+      </c>
+      <c r="G212" s="7">
+        <v>247.33684</v>
       </c>
       <c r="H212">
-        <v>253.86832000000001</v>
+        <v>246.86539999999999</v>
       </c>
       <c r="I212" t="s">
         <v>367</v>
@@ -13837,23 +13839,23 @@
       <c r="J212">
         <v>0</v>
       </c>
-      <c r="K212">
-        <v>255.5487</v>
-      </c>
-      <c r="L212">
-        <v>255.52598599999999</v>
-      </c>
-      <c r="M212" t="s">
-        <v>367</v>
+      <c r="K212" s="7">
+        <v>247.79705999999999</v>
+      </c>
+      <c r="L212" s="2">
+        <v>247.79705999999999</v>
+      </c>
+      <c r="M212">
+        <v>10.145659</v>
       </c>
       <c r="N212">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O212" s="2">
-        <v>200.62246999999999</v>
+        <v>173.25054</v>
       </c>
       <c r="P212" s="2">
-        <v>195.100988</v>
+        <v>165.256564</v>
       </c>
       <c r="Q212" t="s">
         <v>367</v>
@@ -13867,7 +13869,7 @@
         <v>392</v>
       </c>
       <c r="B213" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C213">
         <v>7000</v>
@@ -13876,16 +13878,16 @@
         <v>300</v>
       </c>
       <c r="E213" s="1">
-        <v>1.53294E-3</v>
-      </c>
-      <c r="F213">
-        <v>354.48030999999997</v>
-      </c>
-      <c r="G213">
-        <v>353.82341000000002</v>
+        <v>1.5150999999999999E-3</v>
+      </c>
+      <c r="F213" s="7">
+        <v>336.30565999999999</v>
+      </c>
+      <c r="G213" s="7">
+        <v>335.19159000000002</v>
       </c>
       <c r="H213">
-        <v>352.72425500000003</v>
+        <v>334.34724799999998</v>
       </c>
       <c r="I213" t="s">
         <v>367</v>
@@ -13893,11 +13895,11 @@
       <c r="J213">
         <v>0</v>
       </c>
-      <c r="K213">
-        <v>354.41550000000001</v>
-      </c>
-      <c r="L213">
-        <v>354.26472000000001</v>
+      <c r="K213" s="7">
+        <v>336.12635999999998</v>
+      </c>
+      <c r="L213" s="2">
+        <v>336.00854600000002</v>
       </c>
       <c r="M213" t="s">
         <v>367</v>
@@ -13906,10 +13908,10 @@
         <v>0</v>
       </c>
       <c r="O213" s="2">
-        <v>257.99099000000001</v>
+        <v>233.14454000000001</v>
       </c>
       <c r="P213" s="2">
-        <v>247.200424</v>
+        <v>220.39002600000001</v>
       </c>
       <c r="Q213" t="s">
         <v>367</v>
@@ -13923,7 +13925,7 @@
         <v>392</v>
       </c>
       <c r="B214" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C214">
         <v>7000</v>
@@ -13932,16 +13934,16 @@
         <v>400</v>
       </c>
       <c r="E214" s="1">
-        <v>1.53294E-3</v>
-      </c>
-      <c r="F214">
-        <v>442.89061500000003</v>
-      </c>
-      <c r="G214">
-        <v>440.69545499999998</v>
+        <v>1.5150999999999999E-3</v>
+      </c>
+      <c r="F214" s="7">
+        <v>416.78546999999998</v>
+      </c>
+      <c r="G214" s="7">
+        <v>416.33783</v>
       </c>
       <c r="H214">
-        <v>439.66992399999998</v>
+        <v>414.72527400000001</v>
       </c>
       <c r="I214" t="s">
         <v>367</v>
@@ -13949,11 +13951,11 @@
       <c r="J214">
         <v>0</v>
       </c>
-      <c r="K214">
-        <v>442.62848500000001</v>
-      </c>
-      <c r="L214">
-        <v>442.02394700000002</v>
+      <c r="K214" s="7">
+        <v>416.26258999999999</v>
+      </c>
+      <c r="L214" s="2">
+        <v>416.14019200000001</v>
       </c>
       <c r="M214" t="s">
         <v>367</v>
@@ -13962,10 +13964,10 @@
         <v>0</v>
       </c>
       <c r="O214" s="2">
-        <v>303.73565000000002</v>
+        <v>292.04273999999998</v>
       </c>
       <c r="P214" s="2">
-        <v>294.27895599999999</v>
+        <v>280.86408399999999</v>
       </c>
       <c r="Q214" t="s">
         <v>367</v>
@@ -13979,7 +13981,7 @@
         <v>392</v>
       </c>
       <c r="B215" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="C215">
         <v>7000</v>
@@ -13988,16 +13990,16 @@
         <v>500</v>
       </c>
       <c r="E215" s="1">
-        <v>1.53294E-3</v>
-      </c>
-      <c r="F215">
-        <v>524.15727000000004</v>
-      </c>
-      <c r="G215">
-        <v>522.10491000000002</v>
+        <v>1.5150999999999999E-3</v>
+      </c>
+      <c r="F215" s="7">
+        <v>488.80971</v>
+      </c>
+      <c r="G215" s="7">
+        <v>486.36331999999999</v>
       </c>
       <c r="H215">
-        <v>521.21795799999995</v>
+        <v>485.09733799999998</v>
       </c>
       <c r="I215" t="s">
         <v>367</v>
@@ -14005,11 +14007,11 @@
       <c r="J215">
         <v>0</v>
       </c>
-      <c r="K215">
-        <v>523.66161</v>
-      </c>
-      <c r="L215">
-        <v>523.14984000000004</v>
+      <c r="K215" s="7">
+        <v>487.98117000000002</v>
+      </c>
+      <c r="L215" s="2">
+        <v>487.77013599999998</v>
       </c>
       <c r="M215" t="s">
         <v>367</v>
@@ -14018,10 +14020,10 @@
         <v>0</v>
       </c>
       <c r="O215" s="2">
-        <v>375.50416999999999</v>
+        <v>349.66496000000001</v>
       </c>
       <c r="P215" s="2">
-        <v>364.401656</v>
+        <v>329.18131199999999</v>
       </c>
       <c r="Q215" t="s">
         <v>367</v>
@@ -14035,7 +14037,7 @@
         <v>392</v>
       </c>
       <c r="B216" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C216">
         <v>7000</v>
@@ -14044,16 +14046,16 @@
         <v>100</v>
       </c>
       <c r="E216" s="1">
-        <v>1.5151400000000001E-3</v>
-      </c>
-      <c r="F216">
-        <v>142.13679999999999</v>
-      </c>
-      <c r="G216">
-        <v>142.03421</v>
+        <v>1.4718800000000001E-3</v>
+      </c>
+      <c r="F216" s="7">
+        <v>160.60842</v>
+      </c>
+      <c r="G216" s="7">
+        <v>160.60103000000001</v>
       </c>
       <c r="H216">
-        <v>141.87070800000001</v>
+        <v>160.489194</v>
       </c>
       <c r="I216" t="s">
         <v>367</v>
@@ -14061,23 +14063,23 @@
       <c r="J216">
         <v>0</v>
       </c>
-      <c r="K216">
-        <v>142.13679999999999</v>
-      </c>
-      <c r="L216">
-        <v>142.13679999999999</v>
+      <c r="K216" s="7">
+        <v>160.60842</v>
+      </c>
+      <c r="L216" s="2">
+        <v>160.60842</v>
       </c>
       <c r="M216">
-        <v>3.824681</v>
+        <v>7.2784230000000001</v>
       </c>
       <c r="N216">
         <v>5</v>
       </c>
       <c r="O216" s="2">
-        <v>97.164249999999996</v>
+        <v>132.23325</v>
       </c>
       <c r="P216" s="2">
-        <v>92.234967999999995</v>
+        <v>125.900102</v>
       </c>
       <c r="Q216" t="s">
         <v>367</v>
@@ -14091,7 +14093,7 @@
         <v>392</v>
       </c>
       <c r="B217" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C217">
         <v>7000</v>
@@ -14100,16 +14102,16 @@
         <v>200</v>
       </c>
       <c r="E217" s="1">
-        <v>1.5151400000000001E-3</v>
-      </c>
-      <c r="F217">
-        <v>247.79705999999999</v>
-      </c>
-      <c r="G217">
-        <v>247.14576</v>
+        <v>1.4718800000000001E-3</v>
+      </c>
+      <c r="F217" s="7">
+        <v>282.06218999999999</v>
+      </c>
+      <c r="G217" s="7">
+        <v>281.37416999999999</v>
       </c>
       <c r="H217">
-        <v>246.53982199999999</v>
+        <v>280.71854000000002</v>
       </c>
       <c r="I217" t="s">
         <v>367</v>
@@ -14117,23 +14119,23 @@
       <c r="J217">
         <v>0</v>
       </c>
-      <c r="K217">
-        <v>247.79705999999999</v>
-      </c>
-      <c r="L217">
-        <v>247.59584799999999</v>
-      </c>
-      <c r="M217">
-        <v>25.431833999999998</v>
+      <c r="K217" s="7">
+        <v>281.72043000000002</v>
+      </c>
+      <c r="L217" s="2">
+        <v>281.68038000000001</v>
+      </c>
+      <c r="M217" t="s">
+        <v>367</v>
       </c>
       <c r="N217">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O217" s="2">
-        <v>173.25054</v>
+        <v>227.864</v>
       </c>
       <c r="P217" s="2">
-        <v>165.256564</v>
+        <v>215.60388599999999</v>
       </c>
       <c r="Q217" t="s">
         <v>367</v>
@@ -14147,7 +14149,7 @@
         <v>392</v>
       </c>
       <c r="B218" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C218">
         <v>7000</v>
@@ -14156,16 +14158,16 @@
         <v>300</v>
       </c>
       <c r="E218" s="1">
-        <v>1.5151400000000001E-3</v>
-      </c>
-      <c r="F218">
-        <v>336.30565999999999</v>
-      </c>
-      <c r="G218">
-        <v>334.77213499999999</v>
+        <v>1.4718800000000001E-3</v>
+      </c>
+      <c r="F218" s="7">
+        <v>388.39409000000001</v>
+      </c>
+      <c r="G218" s="7">
+        <v>387.83159999999998</v>
       </c>
       <c r="H218">
-        <v>334.37756400000001</v>
+        <v>386.90218599999997</v>
       </c>
       <c r="I218" t="s">
         <v>367</v>
@@ -14173,11 +14175,11 @@
       <c r="J218">
         <v>0</v>
       </c>
-      <c r="K218">
-        <v>336.20999499999999</v>
-      </c>
-      <c r="L218">
-        <v>335.78627699999998</v>
+      <c r="K218" s="7">
+        <v>388.11849000000001</v>
+      </c>
+      <c r="L218" s="2">
+        <v>388.03724599999998</v>
       </c>
       <c r="M218" t="s">
         <v>367</v>
@@ -14186,10 +14188,10 @@
         <v>0</v>
       </c>
       <c r="O218" s="2">
-        <v>233.14454000000001</v>
+        <v>294.14433000000002</v>
       </c>
       <c r="P218" s="2">
-        <v>220.39002600000001</v>
+        <v>278.52568600000001</v>
       </c>
       <c r="Q218" t="s">
         <v>367</v>
@@ -14203,7 +14205,7 @@
         <v>392</v>
       </c>
       <c r="B219" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C219">
         <v>7000</v>
@@ -14212,16 +14214,16 @@
         <v>400</v>
       </c>
       <c r="E219" s="1">
-        <v>1.5151400000000001E-3</v>
-      </c>
-      <c r="F219">
-        <v>416.79508499999997</v>
-      </c>
-      <c r="G219">
-        <v>415.35574500000001</v>
+        <v>1.4718800000000001E-3</v>
+      </c>
+      <c r="F219" s="7">
+        <v>483.96174999999999</v>
+      </c>
+      <c r="G219" s="7">
+        <v>483.21778</v>
       </c>
       <c r="H219">
-        <v>414.19503700000001</v>
+        <v>482.178606</v>
       </c>
       <c r="I219" t="s">
         <v>367</v>
@@ -14229,11 +14231,11 @@
       <c r="J219">
         <v>0</v>
       </c>
-      <c r="K219">
-        <v>416.27220499999999</v>
-      </c>
-      <c r="L219">
-        <v>415.79192899999998</v>
+      <c r="K219" s="7">
+        <v>483.50227000000001</v>
+      </c>
+      <c r="L219" s="2">
+        <v>483.25977399999999</v>
       </c>
       <c r="M219" t="s">
         <v>367</v>
@@ -14242,10 +14244,10 @@
         <v>0</v>
       </c>
       <c r="O219" s="2">
-        <v>292.04273999999998</v>
+        <v>378.0489</v>
       </c>
       <c r="P219" s="2">
-        <v>280.86408399999999</v>
+        <v>350.63984399999998</v>
       </c>
       <c r="Q219" t="s">
         <v>367</v>
@@ -14259,7 +14261,7 @@
         <v>392</v>
       </c>
       <c r="B220" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C220">
         <v>7000</v>
@@ -14268,16 +14270,16 @@
         <v>500</v>
       </c>
       <c r="E220" s="1">
-        <v>1.5151400000000001E-3</v>
-      </c>
-      <c r="F220">
-        <v>488.81932499999999</v>
-      </c>
-      <c r="G220">
-        <v>486.396795</v>
+        <v>1.4718800000000001E-3</v>
+      </c>
+      <c r="F220" s="7">
+        <v>572.51418999999999</v>
+      </c>
+      <c r="G220" s="7">
+        <v>571.32264999999995</v>
       </c>
       <c r="H220">
-        <v>485.52062699999999</v>
+        <v>570.08389199999999</v>
       </c>
       <c r="I220" t="s">
         <v>367</v>
@@ -14285,11 +14287,11 @@
       <c r="J220">
         <v>0</v>
       </c>
-      <c r="K220">
-        <v>487.824635</v>
-      </c>
-      <c r="L220">
-        <v>487.507881</v>
+      <c r="K220" s="7">
+        <v>572.46213</v>
+      </c>
+      <c r="L220" s="2">
+        <v>572.22895400000004</v>
       </c>
       <c r="M220" t="s">
         <v>367</v>
@@ -14298,10 +14300,10 @@
         <v>0</v>
       </c>
       <c r="O220" s="2">
-        <v>349.66496000000001</v>
+        <v>424.66541999999998</v>
       </c>
       <c r="P220" s="2">
-        <v>329.18131199999999</v>
+        <v>410.54433999999998</v>
       </c>
       <c r="Q220" t="s">
         <v>367</v>
@@ -14315,7 +14317,7 @@
         <v>392</v>
       </c>
       <c r="B221" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C221">
         <v>7000</v>
@@ -14324,40 +14326,40 @@
         <v>100</v>
       </c>
       <c r="E221" s="1">
-        <v>1.47196E-3</v>
-      </c>
-      <c r="F221">
-        <v>160.60842</v>
-      </c>
-      <c r="G221">
-        <v>160.60103000000001</v>
+        <v>1.4577100000000001E-3</v>
+      </c>
+      <c r="F221" s="7">
+        <v>156.42930999999999</v>
+      </c>
+      <c r="G221" s="7">
+        <v>156.42930999999999</v>
       </c>
       <c r="H221">
-        <v>160.215506</v>
-      </c>
-      <c r="I221" t="s">
-        <v>367</v>
+        <v>156.42930999999999</v>
+      </c>
+      <c r="I221">
+        <v>31.992387000000001</v>
       </c>
       <c r="J221">
-        <v>0</v>
-      </c>
-      <c r="K221">
-        <v>160.60842</v>
-      </c>
-      <c r="L221">
-        <v>160.606942</v>
+        <v>5</v>
+      </c>
+      <c r="K221" s="7">
+        <v>156.42930999999999</v>
+      </c>
+      <c r="L221" s="2">
+        <v>156.42930999999999</v>
       </c>
       <c r="M221">
-        <v>22.229817000000001</v>
+        <v>0.124422</v>
       </c>
       <c r="N221">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O221" s="2">
-        <v>132.23325</v>
+        <v>114.87414</v>
       </c>
       <c r="P221" s="2">
-        <v>125.900102</v>
+        <v>110.80799399999999</v>
       </c>
       <c r="Q221" t="s">
         <v>367</v>
@@ -14371,7 +14373,7 @@
         <v>392</v>
       </c>
       <c r="B222" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C222">
         <v>7000</v>
@@ -14380,16 +14382,16 @@
         <v>200</v>
       </c>
       <c r="E222" s="1">
-        <v>1.47196E-3</v>
-      </c>
-      <c r="F222">
-        <v>282.06218999999999</v>
-      </c>
-      <c r="G222">
-        <v>281.16100999999998</v>
+        <v>1.4577100000000001E-3</v>
+      </c>
+      <c r="F222" s="7">
+        <v>266.12285000000003</v>
+      </c>
+      <c r="G222" s="7">
+        <v>264.99907999999999</v>
       </c>
       <c r="H222">
-        <v>280.17756600000001</v>
+        <v>264.76734599999997</v>
       </c>
       <c r="I222" t="s">
         <v>367</v>
@@ -14397,23 +14399,23 @@
       <c r="J222">
         <v>0</v>
       </c>
-      <c r="K222">
-        <v>281.72043000000002</v>
-      </c>
-      <c r="L222">
-        <v>281.60028</v>
-      </c>
-      <c r="M222" t="s">
-        <v>367</v>
+      <c r="K222" s="7">
+        <v>266.12285000000003</v>
+      </c>
+      <c r="L222" s="2">
+        <v>266.12285000000003</v>
+      </c>
+      <c r="M222">
+        <v>15.113811999999999</v>
       </c>
       <c r="N222">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O222" s="2">
-        <v>227.864</v>
+        <v>196.67894000000001</v>
       </c>
       <c r="P222" s="2">
-        <v>215.60388599999999</v>
+        <v>189.78016199999999</v>
       </c>
       <c r="Q222" t="s">
         <v>367</v>
@@ -14427,7 +14429,7 @@
         <v>392</v>
       </c>
       <c r="B223" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C223">
         <v>7000</v>
@@ -14436,16 +14438,16 @@
         <v>300</v>
       </c>
       <c r="E223" s="1">
-        <v>1.47196E-3</v>
-      </c>
-      <c r="F223">
-        <v>388.39409000000001</v>
-      </c>
-      <c r="G223">
-        <v>388.16667000000001</v>
+        <v>1.4577100000000001E-3</v>
+      </c>
+      <c r="F223" s="7">
+        <v>361.99662999999998</v>
+      </c>
+      <c r="G223" s="7">
+        <v>360.57880999999998</v>
       </c>
       <c r="H223">
-        <v>387.01029399999999</v>
+        <v>359.54206199999999</v>
       </c>
       <c r="I223" t="s">
         <v>367</v>
@@ -14453,23 +14455,23 @@
       <c r="J223">
         <v>0</v>
       </c>
-      <c r="K223">
-        <v>388.08981999999997</v>
-      </c>
-      <c r="L223">
-        <v>387.996374</v>
-      </c>
-      <c r="M223" t="s">
-        <v>367</v>
+      <c r="K223" s="7">
+        <v>361.99662999999998</v>
+      </c>
+      <c r="L223" s="2">
+        <v>361.82717200000002</v>
+      </c>
+      <c r="M223">
+        <v>25.470011</v>
       </c>
       <c r="N223">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O223" s="2">
-        <v>294.14433000000002</v>
+        <v>259.30795999999998</v>
       </c>
       <c r="P223" s="2">
-        <v>278.52568600000001</v>
+        <v>248.85695000000001</v>
       </c>
       <c r="Q223" t="s">
         <v>367</v>
@@ -14483,7 +14485,7 @@
         <v>392</v>
       </c>
       <c r="B224" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C224">
         <v>7000</v>
@@ -14492,16 +14494,16 @@
         <v>400</v>
       </c>
       <c r="E224" s="1">
-        <v>1.47196E-3</v>
-      </c>
-      <c r="F224">
-        <v>483.96174999999999</v>
-      </c>
-      <c r="G224">
-        <v>483.28975000000003</v>
+        <v>1.4577100000000001E-3</v>
+      </c>
+      <c r="F224" s="7">
+        <v>446.82528000000002</v>
+      </c>
+      <c r="G224" s="7">
+        <v>446.10257999999999</v>
       </c>
       <c r="H224">
-        <v>482.48890399999999</v>
+        <v>445.01344</v>
       </c>
       <c r="I224" t="s">
         <v>367</v>
@@ -14509,11 +14511,11 @@
       <c r="J224">
         <v>0</v>
       </c>
-      <c r="K224">
-        <v>483.67795999999998</v>
-      </c>
-      <c r="L224">
-        <v>483.42386800000003</v>
+      <c r="K224" s="7">
+        <v>446.54917999999998</v>
+      </c>
+      <c r="L224" s="2">
+        <v>446.35672199999999</v>
       </c>
       <c r="M224" t="s">
         <v>367</v>
@@ -14522,10 +14524,10 @@
         <v>0</v>
       </c>
       <c r="O224" s="2">
-        <v>378.0489</v>
+        <v>313.39211</v>
       </c>
       <c r="P224" s="2">
-        <v>350.63984399999998</v>
+        <v>303.58950199999998</v>
       </c>
       <c r="Q224" t="s">
         <v>367</v>
@@ -14539,7 +14541,7 @@
         <v>392</v>
       </c>
       <c r="B225" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C225">
         <v>7000</v>
@@ -14548,16 +14550,16 @@
         <v>500</v>
       </c>
       <c r="E225" s="1">
-        <v>1.47196E-3</v>
-      </c>
-      <c r="F225">
-        <v>572.51418999999999</v>
-      </c>
-      <c r="G225">
-        <v>571.32974999999999</v>
+        <v>1.4577100000000001E-3</v>
+      </c>
+      <c r="F225" s="7">
+        <v>523.84563000000003</v>
+      </c>
+      <c r="G225" s="7">
+        <v>521.49216999999999</v>
       </c>
       <c r="H225">
-        <v>570.37675999999999</v>
+        <v>520.29437800000005</v>
       </c>
       <c r="I225" t="s">
         <v>367</v>
@@ -14565,11 +14567,11 @@
       <c r="J225">
         <v>0</v>
       </c>
-      <c r="K225">
-        <v>572.04553999999996</v>
-      </c>
-      <c r="L225">
-        <v>571.93580599999996</v>
+      <c r="K225" s="7">
+        <v>523.46379999999999</v>
+      </c>
+      <c r="L225" s="2">
+        <v>522.92005600000005</v>
       </c>
       <c r="M225" t="s">
         <v>367</v>
@@ -14578,10 +14580,10 @@
         <v>0</v>
       </c>
       <c r="O225" s="2">
-        <v>424.66541999999998</v>
+        <v>376.19797</v>
       </c>
       <c r="P225" s="2">
-        <v>410.54433999999998</v>
+        <v>356.58093200000002</v>
       </c>
       <c r="Q225" t="s">
         <v>367</v>
@@ -14595,7 +14597,7 @@
         <v>392</v>
       </c>
       <c r="B226" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C226">
         <v>7000</v>
@@ -14604,40 +14606,40 @@
         <v>100</v>
       </c>
       <c r="E226" s="1">
-        <v>1.45773E-3</v>
-      </c>
-      <c r="F226">
-        <v>156.42930999999999</v>
-      </c>
-      <c r="G226">
-        <v>156.42930999999999</v>
+        <v>1.43804E-3</v>
+      </c>
+      <c r="F226" s="7">
+        <v>129.36341999999999</v>
+      </c>
+      <c r="G226" s="7">
+        <v>128.81952000000001</v>
       </c>
       <c r="H226">
-        <v>156.293104</v>
-      </c>
-      <c r="I226">
-        <v>7.4099130000000004</v>
+        <v>128.58158399999999</v>
+      </c>
+      <c r="I226" t="s">
+        <v>367</v>
       </c>
       <c r="J226">
-        <v>4</v>
-      </c>
-      <c r="K226">
-        <v>156.42930999999999</v>
-      </c>
-      <c r="L226">
-        <v>156.42930999999999</v>
-      </c>
-      <c r="M226">
-        <v>0.50278699999999998</v>
+        <v>0</v>
+      </c>
+      <c r="K226" s="7">
+        <v>128.98062999999999</v>
+      </c>
+      <c r="L226" s="2">
+        <v>128.98062999999999</v>
+      </c>
+      <c r="M226" t="s">
+        <v>367</v>
       </c>
       <c r="N226">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O226" s="2">
-        <v>114.87414</v>
+        <v>107.87851999999999</v>
       </c>
       <c r="P226" s="2">
-        <v>110.80799399999999</v>
+        <v>102.8111</v>
       </c>
       <c r="Q226" t="s">
         <v>367</v>
@@ -14651,7 +14653,7 @@
         <v>392</v>
       </c>
       <c r="B227" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C227">
         <v>7000</v>
@@ -14660,16 +14662,16 @@
         <v>200</v>
       </c>
       <c r="E227" s="1">
-        <v>1.45773E-3</v>
-      </c>
-      <c r="F227">
-        <v>266.12285000000003</v>
-      </c>
-      <c r="G227">
-        <v>265.62203</v>
+        <v>1.43804E-3</v>
+      </c>
+      <c r="F227" s="7">
+        <v>238.34729999999999</v>
+      </c>
+      <c r="G227" s="7">
+        <v>237.55244999999999</v>
       </c>
       <c r="H227">
-        <v>264.78695800000003</v>
+        <v>237.23088000000001</v>
       </c>
       <c r="I227" t="s">
         <v>367</v>
@@ -14677,23 +14679,23 @@
       <c r="J227">
         <v>0</v>
       </c>
-      <c r="K227">
-        <v>266.12285000000003</v>
-      </c>
-      <c r="L227">
-        <v>266.12156199999998</v>
+      <c r="K227" s="7">
+        <v>238.34729999999999</v>
+      </c>
+      <c r="L227" s="2">
+        <v>238.27177599999999</v>
       </c>
       <c r="M227">
-        <v>7.9811909999999999</v>
+        <v>40.619342000000003</v>
       </c>
       <c r="N227">
         <v>4</v>
       </c>
       <c r="O227" s="2">
-        <v>196.67894000000001</v>
+        <v>195.05267000000001</v>
       </c>
       <c r="P227" s="2">
-        <v>189.78016199999999</v>
+        <v>191.34121999999999</v>
       </c>
       <c r="Q227" t="s">
         <v>367</v>
@@ -14707,7 +14709,7 @@
         <v>392</v>
       </c>
       <c r="B228" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C228">
         <v>7000</v>
@@ -14716,16 +14718,16 @@
         <v>300</v>
       </c>
       <c r="E228" s="1">
-        <v>1.45773E-3</v>
-      </c>
-      <c r="F228">
-        <v>361.99662999999998</v>
-      </c>
-      <c r="G228">
-        <v>360.33089000000001</v>
+        <v>1.43804E-3</v>
+      </c>
+      <c r="F228" s="7">
+        <v>337.32862</v>
+      </c>
+      <c r="G228" s="7">
+        <v>336.08528000000001</v>
       </c>
       <c r="H228">
-        <v>359.33782400000001</v>
+        <v>335.62956400000002</v>
       </c>
       <c r="I228" t="s">
         <v>367</v>
@@ -14733,23 +14735,23 @@
       <c r="J228">
         <v>0</v>
       </c>
-      <c r="K228">
-        <v>361.99662999999998</v>
-      </c>
-      <c r="L228">
-        <v>361.74396000000002</v>
-      </c>
-      <c r="M228">
-        <v>8.8765350000000005</v>
+      <c r="K228" s="7">
+        <v>336.96911999999998</v>
+      </c>
+      <c r="L228" s="2">
+        <v>336.813604</v>
+      </c>
+      <c r="M228" t="s">
+        <v>367</v>
       </c>
       <c r="N228">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O228" s="2">
-        <v>259.30795999999998</v>
+        <v>262.94047</v>
       </c>
       <c r="P228" s="2">
-        <v>248.85695000000001</v>
+        <v>244.14046200000001</v>
       </c>
       <c r="Q228" t="s">
         <v>367</v>
@@ -14763,7 +14765,7 @@
         <v>392</v>
       </c>
       <c r="B229" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C229">
         <v>7000</v>
@@ -14772,16 +14774,16 @@
         <v>400</v>
       </c>
       <c r="E229" s="1">
-        <v>1.45773E-3</v>
-      </c>
-      <c r="F229">
-        <v>446.82528000000002</v>
-      </c>
-      <c r="G229">
-        <v>446.38364999999999</v>
+        <v>1.43804E-3</v>
+      </c>
+      <c r="F229" s="7">
+        <v>428.83992000000001</v>
+      </c>
+      <c r="G229" s="7">
+        <v>427.51029999999997</v>
       </c>
       <c r="H229">
-        <v>444.688086</v>
+        <v>426.78179</v>
       </c>
       <c r="I229" t="s">
         <v>367</v>
@@ -14789,11 +14791,11 @@
       <c r="J229">
         <v>0</v>
       </c>
-      <c r="K229">
-        <v>446.65665000000001</v>
-      </c>
-      <c r="L229">
-        <v>446.30169999999998</v>
+      <c r="K229" s="7">
+        <v>428.80497000000003</v>
+      </c>
+      <c r="L229" s="2">
+        <v>428.64142199999998</v>
       </c>
       <c r="M229" t="s">
         <v>367</v>
@@ -14802,10 +14804,10 @@
         <v>0</v>
       </c>
       <c r="O229" s="2">
-        <v>313.39211</v>
+        <v>319.90992</v>
       </c>
       <c r="P229" s="2">
-        <v>303.58950199999998</v>
+        <v>298.86469199999999</v>
       </c>
       <c r="Q229" t="s">
         <v>367</v>
@@ -14819,7 +14821,7 @@
         <v>392</v>
       </c>
       <c r="B230" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C230">
         <v>7000</v>
@@ -14828,16 +14830,16 @@
         <v>500</v>
       </c>
       <c r="E230" s="1">
-        <v>1.45773E-3</v>
-      </c>
-      <c r="F230">
-        <v>523.84563000000003</v>
-      </c>
-      <c r="G230">
-        <v>521.75994000000003</v>
+        <v>1.43804E-3</v>
+      </c>
+      <c r="F230" s="7">
+        <v>511.22753</v>
+      </c>
+      <c r="G230" s="7">
+        <v>509.09719999999999</v>
       </c>
       <c r="H230">
-        <v>521.31202800000005</v>
+        <v>507.79163399999999</v>
       </c>
       <c r="I230" t="s">
         <v>367</v>
@@ -14845,11 +14847,11 @@
       <c r="J230">
         <v>0</v>
       </c>
-      <c r="K230">
-        <v>523.15422999999998</v>
-      </c>
-      <c r="L230">
-        <v>522.54365600000006</v>
+      <c r="K230" s="7">
+        <v>510.97777000000002</v>
+      </c>
+      <c r="L230" s="2">
+        <v>510.77173599999998</v>
       </c>
       <c r="M230" t="s">
         <v>367</v>
@@ -14858,10 +14860,10 @@
         <v>0</v>
       </c>
       <c r="O230" s="2">
-        <v>376.19797</v>
+        <v>361.03273000000002</v>
       </c>
       <c r="P230" s="2">
-        <v>356.58093200000002</v>
+        <v>354.11626000000001</v>
       </c>
       <c r="Q230" t="s">
         <v>367</v>
@@ -14875,7 +14877,7 @@
         <v>392</v>
       </c>
       <c r="B231" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C231">
         <v>7000</v>
@@ -14884,40 +14886,40 @@
         <v>100</v>
       </c>
       <c r="E231" s="1">
-        <v>1.43808E-3</v>
-      </c>
-      <c r="F231">
-        <v>129.36341999999999</v>
-      </c>
-      <c r="G231">
-        <v>128.79311999999999</v>
+        <v>1.5466900000000001E-3</v>
+      </c>
+      <c r="F231" s="7">
+        <v>147.21297999999999</v>
+      </c>
+      <c r="G231" s="7">
+        <v>147.21297999999999</v>
       </c>
       <c r="H231">
-        <v>128.46249</v>
-      </c>
-      <c r="I231" t="s">
-        <v>367</v>
+        <v>147.184752</v>
+      </c>
+      <c r="I231">
+        <v>17.282883000000002</v>
       </c>
       <c r="J231">
-        <v>0</v>
-      </c>
-      <c r="K231">
-        <v>128.98062999999999</v>
-      </c>
-      <c r="L231">
-        <v>128.98062999999999</v>
-      </c>
-      <c r="M231" t="s">
-        <v>367</v>
+        <v>4</v>
+      </c>
+      <c r="K231" s="7">
+        <v>147.21297999999999</v>
+      </c>
+      <c r="L231" s="2">
+        <v>147.21297999999999</v>
+      </c>
+      <c r="M231">
+        <v>1.4494750000000001</v>
       </c>
       <c r="N231">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O231" s="2">
-        <v>107.87851999999999</v>
+        <v>113.53071</v>
       </c>
       <c r="P231" s="2">
-        <v>102.8111</v>
+        <v>111.149196</v>
       </c>
       <c r="Q231" t="s">
         <v>367</v>
@@ -14931,7 +14933,7 @@
         <v>392</v>
       </c>
       <c r="B232" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C232">
         <v>7000</v>
@@ -14940,16 +14942,16 @@
         <v>200</v>
       </c>
       <c r="E232" s="1">
-        <v>1.43808E-3</v>
-      </c>
-      <c r="F232">
-        <v>238.34729999999999</v>
-      </c>
-      <c r="G232">
-        <v>237.47512</v>
+        <v>1.5466900000000001E-3</v>
+      </c>
+      <c r="F232" s="7">
+        <v>256.88351</v>
+      </c>
+      <c r="G232" s="7">
+        <v>256.81580000000002</v>
       </c>
       <c r="H232">
-        <v>237.008892</v>
+        <v>256.514926</v>
       </c>
       <c r="I232" t="s">
         <v>367</v>
@@ -14957,23 +14959,23 @@
       <c r="J232">
         <v>0</v>
       </c>
-      <c r="K232">
-        <v>238.34729999999999</v>
-      </c>
-      <c r="L232">
-        <v>238.226294</v>
+      <c r="K232" s="7">
+        <v>256.88351</v>
+      </c>
+      <c r="L232" s="2">
+        <v>256.86658999999997</v>
       </c>
       <c r="M232">
-        <v>31.621143</v>
+        <v>41.127676000000001</v>
       </c>
       <c r="N232">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O232" s="2">
-        <v>195.05267000000001</v>
+        <v>217.47901999999999</v>
       </c>
       <c r="P232" s="2">
-        <v>191.34121999999999</v>
+        <v>188.74712199999999</v>
       </c>
       <c r="Q232" t="s">
         <v>367</v>
@@ -14987,7 +14989,7 @@
         <v>392</v>
       </c>
       <c r="B233" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C233">
         <v>7000</v>
@@ -14996,16 +14998,16 @@
         <v>300</v>
       </c>
       <c r="E233" s="1">
-        <v>1.43808E-3</v>
-      </c>
-      <c r="F233">
-        <v>337.32862</v>
-      </c>
-      <c r="G233">
-        <v>336.58855</v>
+        <v>1.5466900000000001E-3</v>
+      </c>
+      <c r="F233" s="7">
+        <v>351.50053000000003</v>
+      </c>
+      <c r="G233" s="7">
+        <v>350.27321000000001</v>
       </c>
       <c r="H233">
-        <v>335.84592800000001</v>
+        <v>349.76402400000001</v>
       </c>
       <c r="I233" t="s">
         <v>367</v>
@@ -15013,11 +15015,11 @@
       <c r="J233">
         <v>0</v>
       </c>
-      <c r="K233">
-        <v>336.93103000000002</v>
-      </c>
-      <c r="L233">
-        <v>336.75477999999998</v>
+      <c r="K233" s="7">
+        <v>351.44675000000001</v>
+      </c>
+      <c r="L233" s="2">
+        <v>351.23800199999999</v>
       </c>
       <c r="M233" t="s">
         <v>367</v>
@@ -15026,10 +15028,10 @@
         <v>0</v>
       </c>
       <c r="O233" s="2">
-        <v>262.94047</v>
+        <v>247.66099</v>
       </c>
       <c r="P233" s="2">
-        <v>244.14046200000001</v>
+        <v>241.229782</v>
       </c>
       <c r="Q233" t="s">
         <v>367</v>
@@ -15043,7 +15045,7 @@
         <v>392</v>
       </c>
       <c r="B234" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C234">
         <v>7000</v>
@@ -15052,16 +15054,16 @@
         <v>400</v>
       </c>
       <c r="E234" s="1">
-        <v>1.43808E-3</v>
-      </c>
-      <c r="F234">
-        <v>428.83992000000001</v>
-      </c>
-      <c r="G234">
-        <v>427.41764999999998</v>
+        <v>1.5466900000000001E-3</v>
+      </c>
+      <c r="F234" s="7">
+        <v>438.72872999999998</v>
+      </c>
+      <c r="G234" s="7">
+        <v>437.07792999999998</v>
       </c>
       <c r="H234">
-        <v>426.77555799999999</v>
+        <v>436.35433799999998</v>
       </c>
       <c r="I234" t="s">
         <v>367</v>
@@ -15069,23 +15071,23 @@
       <c r="J234">
         <v>0</v>
       </c>
-      <c r="K234">
-        <v>428.83992000000001</v>
-      </c>
-      <c r="L234">
-        <v>428.66596800000002</v>
-      </c>
-      <c r="M234">
-        <v>44.995258</v>
+      <c r="K234" s="7">
+        <v>438.15688999999998</v>
+      </c>
+      <c r="L234" s="2">
+        <v>437.86635799999999</v>
+      </c>
+      <c r="M234" t="s">
+        <v>367</v>
       </c>
       <c r="N234">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O234" s="2">
-        <v>319.90992</v>
+        <v>326.48577</v>
       </c>
       <c r="P234" s="2">
-        <v>298.86469199999999</v>
+        <v>300.42398800000001</v>
       </c>
       <c r="Q234" t="s">
         <v>367</v>
@@ -15099,7 +15101,7 @@
         <v>392</v>
       </c>
       <c r="B235" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="C235">
         <v>7000</v>
@@ -15108,16 +15110,16 @@
         <v>500</v>
       </c>
       <c r="E235" s="1">
-        <v>1.43808E-3</v>
-      </c>
-      <c r="F235">
-        <v>511.22753</v>
-      </c>
-      <c r="G235">
-        <v>509.27987000000002</v>
+        <v>1.5466900000000001E-3</v>
+      </c>
+      <c r="F235" s="7">
+        <v>520.36280999999997</v>
+      </c>
+      <c r="G235" s="7">
+        <v>518.34614999999997</v>
       </c>
       <c r="H235">
-        <v>507.820786</v>
+        <v>516.82395399999996</v>
       </c>
       <c r="I235" t="s">
         <v>367</v>
@@ -15125,11 +15127,11 @@
       <c r="J235">
         <v>0</v>
       </c>
-      <c r="K235">
-        <v>511.12373000000002</v>
-      </c>
-      <c r="L235">
-        <v>510.97776599999997</v>
+      <c r="K235" s="7">
+        <v>520.20045000000005</v>
+      </c>
+      <c r="L235" s="2">
+        <v>519.81827999999996</v>
       </c>
       <c r="M235" t="s">
         <v>367</v>
@@ -15138,10 +15140,10 @@
         <v>0</v>
       </c>
       <c r="O235" s="2">
-        <v>361.03273000000002</v>
+        <v>379.45794999999998</v>
       </c>
       <c r="P235" s="2">
-        <v>352.80276600000002</v>
+        <v>367.57217600000001</v>
       </c>
       <c r="Q235" t="s">
         <v>367</v>
@@ -15155,7 +15157,7 @@
         <v>392</v>
       </c>
       <c r="B236" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C236">
         <v>7000</v>
@@ -15164,40 +15166,40 @@
         <v>100</v>
       </c>
       <c r="E236" s="1">
-        <v>1.5468599999999999E-3</v>
-      </c>
-      <c r="F236">
-        <v>147.21297999999999</v>
-      </c>
-      <c r="G236">
-        <v>147.21297999999999</v>
+        <v>1.43151E-3</v>
+      </c>
+      <c r="F236" s="7">
+        <v>140.00452999999999</v>
+      </c>
+      <c r="G236" s="7">
+        <v>140.00452999999999</v>
       </c>
       <c r="H236">
-        <v>147.17847599999999</v>
+        <v>139.97006200000001</v>
       </c>
       <c r="I236">
-        <v>22.722314999999998</v>
+        <v>30.233725</v>
       </c>
       <c r="J236">
-        <v>4</v>
-      </c>
-      <c r="K236">
-        <v>147.21297999999999</v>
-      </c>
-      <c r="L236">
-        <v>147.21297999999999</v>
+        <v>2</v>
+      </c>
+      <c r="K236" s="7">
+        <v>140.00452999999999</v>
+      </c>
+      <c r="L236" s="2">
+        <v>140.00452999999999</v>
       </c>
       <c r="M236">
-        <v>0.83604000000000001</v>
+        <v>4.022411</v>
       </c>
       <c r="N236">
         <v>5</v>
       </c>
       <c r="O236" s="2">
-        <v>113.53071</v>
+        <v>112.75433</v>
       </c>
       <c r="P236" s="2">
-        <v>111.149196</v>
+        <v>106.000338</v>
       </c>
       <c r="Q236" t="s">
         <v>367</v>
@@ -15211,7 +15213,7 @@
         <v>392</v>
       </c>
       <c r="B237" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="C237">
         <v>7000</v>
@@ -15220,16 +15222,16 @@
         <v>200</v>
       </c>
       <c r="E237" s="1">
-        <v>1.5468599999999999E-3</v>
-      </c>
-      <c r="F237">
-        <v>256.88351</v>
-      </c>
-      <c r="G237">
-        <v>256.63941999999997</v>
+        <v>1.43151E-3</v>
+      </c>
+      <c r="F237" s="7">
+        <v>247.84585000000001</v>
+      </c>
+      <c r="G237" s="7">
+        <v>247.76258000000001</v>
       </c>
       <c r="H237">
-        <v>256.37202400000001</v>
+        <v>247.484058</v>
       </c>
       <c r="I237" t="s">
         <v>367</v>
@@ -15237,23 +15239,23 @@
       <c r="J237">
         <v>0</v>
       </c>
-      <c r="K237">
-        <v>256.88351</v>
-      </c>
-      <c r="L237">
-        <v>256.87337600000001</v>
+      <c r="K237" s="7">
+        <v>247.84585000000001</v>
+      </c>
+      <c r="L237" s="2">
+        <v>247.826042</v>
       </c>
       <c r="M237">
-        <v>18.803170000000001</v>
+        <v>10.938629000000001</v>
       </c>
       <c r="N237">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O237" s="2">
-        <v>217.47901999999999</v>
+        <v>191.00614999999999</v>
       </c>
       <c r="P237" s="2">
-        <v>188.74712199999999</v>
+        <v>176.892144</v>
       </c>
       <c r="Q237" t="s">
         <v>367</v>
@@ -15267,7 +15269,7 @@
         <v>392</v>
       </c>
       <c r="B238" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C238">
         <v>7000</v>
@@ -15276,16 +15278,16 @@
         <v>300</v>
       </c>
       <c r="E238" s="1">
-        <v>1.5468599999999999E-3</v>
-      </c>
-      <c r="F238">
-        <v>351.50053000000003</v>
-      </c>
-      <c r="G238">
-        <v>350.43957</v>
+        <v>1.43151E-3</v>
+      </c>
+      <c r="F238" s="7">
+        <v>338.79363000000001</v>
+      </c>
+      <c r="G238" s="7">
+        <v>337.77825999999999</v>
       </c>
       <c r="H238">
-        <v>349.757338</v>
+        <v>337.10023799999999</v>
       </c>
       <c r="I238" t="s">
         <v>367</v>
@@ -15293,23 +15295,23 @@
       <c r="J238">
         <v>0</v>
       </c>
-      <c r="K238">
-        <v>351.44675000000001</v>
-      </c>
-      <c r="L238">
-        <v>351.253244</v>
-      </c>
-      <c r="M238" t="s">
-        <v>367</v>
+      <c r="K238" s="7">
+        <v>338.79363000000001</v>
+      </c>
+      <c r="L238" s="2">
+        <v>338.402286</v>
+      </c>
+      <c r="M238">
+        <v>14.330735000000001</v>
       </c>
       <c r="N238">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O238" s="2">
-        <v>247.66099</v>
+        <v>252.26052999999999</v>
       </c>
       <c r="P238" s="2">
-        <v>241.229782</v>
+        <v>239.114664</v>
       </c>
       <c r="Q238" t="s">
         <v>367</v>
@@ -15323,7 +15325,7 @@
         <v>392</v>
       </c>
       <c r="B239" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="C239">
         <v>7000</v>
@@ -15332,16 +15334,16 @@
         <v>400</v>
       </c>
       <c r="E239" s="1">
-        <v>1.5468599999999999E-3</v>
-      </c>
-      <c r="F239">
-        <v>438.72872999999998</v>
-      </c>
-      <c r="G239">
-        <v>437.44524999999999</v>
+        <v>1.43151E-3</v>
+      </c>
+      <c r="F239" s="7">
+        <v>419.42606999999998</v>
+      </c>
+      <c r="G239" s="7">
+        <v>417.01681000000002</v>
       </c>
       <c r="H239">
-        <v>436.326908</v>
+        <v>416.28735</v>
       </c>
       <c r="I239" t="s">
         <v>367</v>
@@ -15349,11 +15351,11 @@
       <c r="J239">
         <v>0</v>
       </c>
-      <c r="K239">
-        <v>438.15708000000001</v>
-      </c>
-      <c r="L239">
-        <v>437.93005199999999</v>
+      <c r="K239" s="7">
+        <v>419.19886000000002</v>
+      </c>
+      <c r="L239" s="2">
+        <v>418.796806</v>
       </c>
       <c r="M239" t="s">
         <v>367</v>
@@ -15362,10 +15364,10 @@
         <v>0</v>
       </c>
       <c r="O239" s="2">
-        <v>326.48577</v>
+        <v>293.32414</v>
       </c>
       <c r="P239" s="2">
-        <v>300.42398800000001</v>
+        <v>282.34068400000001</v>
       </c>
       <c r="Q239" t="s">
         <v>367</v>
@@ -15379,7 +15381,7 @@
         <v>392</v>
       </c>
       <c r="B240" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C240">
         <v>7000</v>
@@ -15388,16 +15390,16 @@
         <v>500</v>
       </c>
       <c r="E240" s="1">
-        <v>1.5468599999999999E-3</v>
-      </c>
-      <c r="F240">
-        <v>520.36280999999997</v>
-      </c>
-      <c r="G240">
-        <v>518.34488999999996</v>
+        <v>1.43151E-3</v>
+      </c>
+      <c r="F240" s="7">
+        <v>494.06198999999998</v>
+      </c>
+      <c r="G240" s="7">
+        <v>492.92237999999998</v>
       </c>
       <c r="H240">
-        <v>516.53891399999998</v>
+        <v>491.379254</v>
       </c>
       <c r="I240" t="s">
         <v>367</v>
@@ -15405,11 +15407,11 @@
       <c r="J240">
         <v>0</v>
       </c>
-      <c r="K240">
-        <v>519.96007999999995</v>
-      </c>
-      <c r="L240">
-        <v>519.51113199999998</v>
+      <c r="K240" s="7">
+        <v>493.52073000000001</v>
+      </c>
+      <c r="L240" s="2">
+        <v>493.12885999999997</v>
       </c>
       <c r="M240" t="s">
         <v>367</v>
@@ -15418,10 +15420,10 @@
         <v>0</v>
       </c>
       <c r="O240" s="2">
-        <v>379.45794999999998</v>
+        <v>380.15454999999997</v>
       </c>
       <c r="P240" s="2">
-        <v>367.57217600000001</v>
+        <v>360.83122800000001</v>
       </c>
       <c r="Q240" t="s">
         <v>367</v>
@@ -15435,7 +15437,7 @@
         <v>392</v>
       </c>
       <c r="B241" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C241">
         <v>7000</v>
@@ -15444,40 +15446,40 @@
         <v>100</v>
       </c>
       <c r="E241" s="1">
-        <v>1.4316699999999999E-3</v>
-      </c>
-      <c r="F241">
-        <v>140.00452999999999</v>
-      </c>
-      <c r="G241">
-        <v>139.85902999999999</v>
+        <v>1.5036699999999999E-3</v>
+      </c>
+      <c r="F241" s="7">
+        <v>161.7431</v>
+      </c>
+      <c r="G241" s="7">
+        <v>161.7431</v>
       </c>
       <c r="H241">
-        <v>139.850538</v>
-      </c>
-      <c r="I241" t="s">
-        <v>367</v>
+        <v>161.586772</v>
+      </c>
+      <c r="I241">
+        <v>14.845529000000001</v>
       </c>
       <c r="J241">
-        <v>0</v>
-      </c>
-      <c r="K241">
-        <v>140.00452999999999</v>
-      </c>
-      <c r="L241">
-        <v>140.00452999999999</v>
+        <v>4</v>
+      </c>
+      <c r="K241" s="7">
+        <v>161.7431</v>
+      </c>
+      <c r="L241" s="2">
+        <v>161.7431</v>
       </c>
       <c r="M241">
-        <v>7.3458170000000003</v>
+        <v>5.5432000000000002E-2</v>
       </c>
       <c r="N241">
         <v>5</v>
       </c>
       <c r="O241" s="2">
-        <v>112.75433</v>
+        <v>114.07156999999999</v>
       </c>
       <c r="P241" s="2">
-        <v>106.000338</v>
+        <v>108.546684</v>
       </c>
       <c r="Q241" t="s">
         <v>367</v>
@@ -15491,7 +15493,7 @@
         <v>392</v>
       </c>
       <c r="B242" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C242">
         <v>7000</v>
@@ -15500,16 +15502,16 @@
         <v>200</v>
       </c>
       <c r="E242" s="1">
-        <v>1.4316699999999999E-3</v>
-      </c>
-      <c r="F242">
-        <v>247.84585000000001</v>
-      </c>
-      <c r="G242">
-        <v>247.68423999999999</v>
+        <v>1.5036699999999999E-3</v>
+      </c>
+      <c r="F242" s="7">
+        <v>285.37745999999999</v>
+      </c>
+      <c r="G242" s="7">
+        <v>285.08262999999999</v>
       </c>
       <c r="H242">
-        <v>247.39899199999999</v>
+        <v>284.12598400000002</v>
       </c>
       <c r="I242" t="s">
         <v>367</v>
@@ -15517,23 +15519,23 @@
       <c r="J242">
         <v>0</v>
       </c>
-      <c r="K242">
-        <v>247.84585000000001</v>
-      </c>
-      <c r="L242">
-        <v>247.803718</v>
+      <c r="K242" s="7">
+        <v>285.37745999999999</v>
+      </c>
+      <c r="L242" s="2">
+        <v>285.36749200000003</v>
       </c>
       <c r="M242">
-        <v>43.056511</v>
+        <v>17.195401</v>
       </c>
       <c r="N242">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O242" s="2">
-        <v>191.00614999999999</v>
+        <v>202.87291999999999</v>
       </c>
       <c r="P242" s="2">
-        <v>176.892144</v>
+        <v>194.13234800000001</v>
       </c>
       <c r="Q242" t="s">
         <v>367</v>
@@ -15547,7 +15549,7 @@
         <v>392</v>
       </c>
       <c r="B243" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C243">
         <v>7000</v>
@@ -15556,16 +15558,16 @@
         <v>300</v>
       </c>
       <c r="E243" s="1">
-        <v>1.4316699999999999E-3</v>
-      </c>
-      <c r="F243">
-        <v>338.79363000000001</v>
-      </c>
-      <c r="G243">
-        <v>338.38380999999998</v>
+        <v>1.5036699999999999E-3</v>
+      </c>
+      <c r="F243" s="7">
+        <v>390.66397000000001</v>
+      </c>
+      <c r="G243" s="7">
+        <v>389.07109000000003</v>
       </c>
       <c r="H243">
-        <v>337.14440000000002</v>
+        <v>388.72413399999999</v>
       </c>
       <c r="I243" t="s">
         <v>367</v>
@@ -15573,23 +15575,23 @@
       <c r="J243">
         <v>0</v>
       </c>
-      <c r="K243">
-        <v>338.79363000000001</v>
-      </c>
-      <c r="L243">
-        <v>338.64009600000003</v>
-      </c>
-      <c r="M243">
-        <v>24.907036000000002</v>
+      <c r="K243" s="7">
+        <v>390.24353000000002</v>
+      </c>
+      <c r="L243" s="2">
+        <v>390.11005999999998</v>
+      </c>
+      <c r="M243" t="s">
+        <v>367</v>
       </c>
       <c r="N243">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O243" s="2">
-        <v>252.26052999999999</v>
+        <v>272.95778999999999</v>
       </c>
       <c r="P243" s="2">
-        <v>239.114664</v>
+        <v>261.17338799999999</v>
       </c>
       <c r="Q243" t="s">
         <v>367</v>
@@ -15603,7 +15605,7 @@
         <v>392</v>
       </c>
       <c r="B244" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C244">
         <v>7000</v>
@@ -15612,16 +15614,16 @@
         <v>400</v>
       </c>
       <c r="E244" s="1">
-        <v>1.4316699999999999E-3</v>
-      </c>
-      <c r="F244">
-        <v>419.42606999999998</v>
-      </c>
-      <c r="G244">
-        <v>417.48181</v>
+        <v>1.5036699999999999E-3</v>
+      </c>
+      <c r="F244" s="7">
+        <v>485.51931999999999</v>
+      </c>
+      <c r="G244" s="7">
+        <v>483.50990000000002</v>
       </c>
       <c r="H244">
-        <v>416.27263799999997</v>
+        <v>482.97663</v>
       </c>
       <c r="I244" t="s">
         <v>367</v>
@@ -15629,11 +15631,11 @@
       <c r="J244">
         <v>0</v>
       </c>
-      <c r="K244">
-        <v>418.8999</v>
-      </c>
-      <c r="L244">
-        <v>418.72498400000001</v>
+      <c r="K244" s="7">
+        <v>485.08031999999997</v>
+      </c>
+      <c r="L244" s="2">
+        <v>484.88711799999999</v>
       </c>
       <c r="M244" t="s">
         <v>367</v>
@@ -15642,10 +15644,10 @@
         <v>0</v>
       </c>
       <c r="O244" s="2">
-        <v>293.32414</v>
+        <v>365.34737000000001</v>
       </c>
       <c r="P244" s="2">
-        <v>282.34068400000001</v>
+        <v>326.52769999999998</v>
       </c>
       <c r="Q244" t="s">
         <v>367</v>
@@ -15659,7 +15661,7 @@
         <v>392</v>
       </c>
       <c r="B245" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="C245">
         <v>7000</v>
@@ -15668,16 +15670,16 @@
         <v>500</v>
       </c>
       <c r="E245" s="1">
-        <v>1.4316699999999999E-3</v>
-      </c>
-      <c r="F245">
-        <v>494.06198999999998</v>
-      </c>
-      <c r="G245">
-        <v>492.44011999999998</v>
+        <v>1.5036699999999999E-3</v>
+      </c>
+      <c r="F245" s="7">
+        <v>572.19514000000004</v>
+      </c>
+      <c r="G245" s="7">
+        <v>571.32731999999999</v>
       </c>
       <c r="H245">
-        <v>491.27867600000002</v>
+        <v>569.55937400000005</v>
       </c>
       <c r="I245" t="s">
         <v>367</v>
@@ -15685,11 +15687,11 @@
       <c r="J245">
         <v>0</v>
       </c>
-      <c r="K245">
-        <v>493.46212000000003</v>
-      </c>
-      <c r="L245">
-        <v>493.07862799999998</v>
+      <c r="K245" s="7">
+        <v>571.69277</v>
+      </c>
+      <c r="L245" s="2">
+        <v>571.36655800000005</v>
       </c>
       <c r="M245" t="s">
         <v>367</v>
@@ -15698,10 +15700,10 @@
         <v>0</v>
       </c>
       <c r="O245" s="2">
-        <v>380.15454999999997</v>
+        <v>394.62335000000002</v>
       </c>
       <c r="P245" s="2">
-        <v>360.83122800000001</v>
+        <v>384.203236</v>
       </c>
       <c r="Q245" t="s">
         <v>367</v>
@@ -15715,7 +15717,7 @@
         <v>392</v>
       </c>
       <c r="B246" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C246">
         <v>7000</v>
@@ -15724,40 +15726,40 @@
         <v>100</v>
       </c>
       <c r="E246" s="1">
-        <v>1.50373E-3</v>
-      </c>
-      <c r="F246">
-        <v>161.7431</v>
-      </c>
-      <c r="G246">
-        <v>161.7431</v>
+        <v>1.5784900000000001E-3</v>
+      </c>
+      <c r="F246" s="7">
+        <v>147.46025</v>
+      </c>
+      <c r="G246" s="7">
+        <v>147.46025</v>
       </c>
       <c r="H246">
-        <v>161.05237199999999</v>
+        <v>147.309606</v>
       </c>
       <c r="I246">
-        <v>46.228766</v>
+        <v>13.565963999999999</v>
       </c>
       <c r="J246">
-        <v>1</v>
-      </c>
-      <c r="K246">
-        <v>161.7431</v>
-      </c>
-      <c r="L246">
-        <v>161.7431</v>
+        <v>4</v>
+      </c>
+      <c r="K246" s="7">
+        <v>147.46025</v>
+      </c>
+      <c r="L246" s="2">
+        <v>147.46025</v>
       </c>
       <c r="M246">
-        <v>0.116628</v>
+        <v>0.15137300000000001</v>
       </c>
       <c r="N246">
         <v>5</v>
       </c>
       <c r="O246" s="2">
-        <v>114.07156999999999</v>
+        <v>119.34896000000001</v>
       </c>
       <c r="P246" s="2">
-        <v>108.546684</v>
+        <v>115.65856599999999</v>
       </c>
       <c r="Q246" t="s">
         <v>367</v>
@@ -15771,7 +15773,7 @@
         <v>392</v>
       </c>
       <c r="B247" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C247">
         <v>7000</v>
@@ -15780,40 +15782,40 @@
         <v>200</v>
       </c>
       <c r="E247" s="1">
-        <v>1.50373E-3</v>
-      </c>
-      <c r="F247">
-        <v>285.37745999999999</v>
-      </c>
-      <c r="G247">
-        <v>285.37745999999999</v>
+        <v>1.5784900000000001E-3</v>
+      </c>
+      <c r="F247" s="7">
+        <v>256.29746</v>
+      </c>
+      <c r="G247" s="7">
+        <v>255.92662000000001</v>
       </c>
       <c r="H247">
-        <v>284.56900400000001</v>
-      </c>
-      <c r="I247">
-        <v>6.471571</v>
+        <v>255.61946800000001</v>
+      </c>
+      <c r="I247" t="s">
+        <v>367</v>
       </c>
       <c r="J247">
-        <v>1</v>
-      </c>
-      <c r="K247">
-        <v>285.37745999999999</v>
-      </c>
-      <c r="L247">
-        <v>285.37745999999999</v>
+        <v>0</v>
+      </c>
+      <c r="K247" s="7">
+        <v>256.29746</v>
+      </c>
+      <c r="L247" s="2">
+        <v>256.26906000000002</v>
       </c>
       <c r="M247">
-        <v>6.3148140000000001</v>
+        <v>18.806948999999999</v>
       </c>
       <c r="N247">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O247" s="2">
-        <v>202.87291999999999</v>
+        <v>198.96678</v>
       </c>
       <c r="P247" s="2">
-        <v>194.13234800000001</v>
+        <v>188.087132</v>
       </c>
       <c r="Q247" t="s">
         <v>367</v>
@@ -15827,7 +15829,7 @@
         <v>392</v>
       </c>
       <c r="B248" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C248">
         <v>7000</v>
@@ -15836,16 +15838,16 @@
         <v>300</v>
       </c>
       <c r="E248" s="1">
-        <v>1.50373E-3</v>
-      </c>
-      <c r="F248">
-        <v>390.66397000000001</v>
-      </c>
-      <c r="G248">
-        <v>389.47016000000002</v>
+        <v>1.5784900000000001E-3</v>
+      </c>
+      <c r="F248" s="7">
+        <v>350.39949999999999</v>
+      </c>
+      <c r="G248" s="7">
+        <v>349.88108999999997</v>
       </c>
       <c r="H248">
-        <v>388.53235999999998</v>
+        <v>349.34956399999999</v>
       </c>
       <c r="I248" t="s">
         <v>367</v>
@@ -15853,11 +15855,11 @@
       <c r="J248">
         <v>0</v>
       </c>
-      <c r="K248">
-        <v>390.02454999999998</v>
-      </c>
-      <c r="L248">
-        <v>389.92920800000002</v>
+      <c r="K248" s="7">
+        <v>350.32562000000001</v>
+      </c>
+      <c r="L248" s="2">
+        <v>350.04558400000002</v>
       </c>
       <c r="M248" t="s">
         <v>367</v>
@@ -15866,10 +15868,10 @@
         <v>0</v>
       </c>
       <c r="O248" s="2">
-        <v>272.95778999999999</v>
+        <v>267.4271</v>
       </c>
       <c r="P248" s="2">
-        <v>261.17338799999999</v>
+        <v>250.31087199999999</v>
       </c>
       <c r="Q248" t="s">
         <v>367</v>
@@ -15883,7 +15885,7 @@
         <v>392</v>
       </c>
       <c r="B249" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="C249">
         <v>7000</v>
@@ -15892,16 +15894,16 @@
         <v>400</v>
       </c>
       <c r="E249" s="1">
-        <v>1.50373E-3</v>
-      </c>
-      <c r="F249">
-        <v>485.51931999999999</v>
-      </c>
-      <c r="G249">
-        <v>483.26459999999997</v>
+        <v>1.5784900000000001E-3</v>
+      </c>
+      <c r="F249" s="7">
+        <v>435.43218000000002</v>
+      </c>
+      <c r="G249" s="7">
+        <v>433.68650000000002</v>
       </c>
       <c r="H249">
-        <v>482.49301200000002</v>
+        <v>432.94922000000003</v>
       </c>
       <c r="I249" t="s">
         <v>367</v>
@@ -15909,11 +15911,11 @@
       <c r="J249">
         <v>0</v>
       </c>
-      <c r="K249">
-        <v>485.29138</v>
-      </c>
-      <c r="L249">
-        <v>485.01092199999999</v>
+      <c r="K249" s="7">
+        <v>435.32171</v>
+      </c>
+      <c r="L249" s="2">
+        <v>435.05330800000002</v>
       </c>
       <c r="M249" t="s">
         <v>367</v>
@@ -15922,10 +15924,10 @@
         <v>0</v>
       </c>
       <c r="O249" s="2">
-        <v>365.34737000000001</v>
+        <v>314.36304000000001</v>
       </c>
       <c r="P249" s="2">
-        <v>326.52769999999998</v>
+        <v>303.00376</v>
       </c>
       <c r="Q249" t="s">
         <v>367</v>
@@ -15939,7 +15941,7 @@
         <v>392</v>
       </c>
       <c r="B250" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C250">
         <v>7000</v>
@@ -15948,16 +15950,16 @@
         <v>500</v>
       </c>
       <c r="E250" s="1">
-        <v>1.50373E-3</v>
-      </c>
-      <c r="F250">
-        <v>572.19514000000004</v>
-      </c>
-      <c r="G250">
-        <v>571.18679999999995</v>
+        <v>1.5784900000000001E-3</v>
+      </c>
+      <c r="F250" s="7">
+        <v>512.72307999999998</v>
+      </c>
+      <c r="G250" s="7">
+        <v>510.50017000000003</v>
       </c>
       <c r="H250">
-        <v>569.81491200000005</v>
+        <v>509.44511999999997</v>
       </c>
       <c r="I250" t="s">
         <v>367</v>
@@ -15965,11 +15967,11 @@
       <c r="J250">
         <v>0</v>
       </c>
-      <c r="K250">
-        <v>571.38815</v>
-      </c>
-      <c r="L250">
-        <v>571.191776</v>
+      <c r="K250" s="7">
+        <v>512.23825999999997</v>
+      </c>
+      <c r="L250" s="2">
+        <v>511.95080000000002</v>
       </c>
       <c r="M250" t="s">
         <v>367</v>
@@ -15978,10 +15980,10 @@
         <v>0</v>
       </c>
       <c r="O250" s="2">
-        <v>394.62335000000002</v>
+        <v>379.13231999999999</v>
       </c>
       <c r="P250" s="2">
-        <v>384.203236</v>
+        <v>356.768214</v>
       </c>
       <c r="Q250" t="s">
         <v>367</v>
@@ -15995,7 +15997,7 @@
         <v>392</v>
       </c>
       <c r="B251" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="C251">
         <v>7000</v>
@@ -16004,40 +16006,40 @@
         <v>100</v>
       </c>
       <c r="E251" s="1">
-        <v>1.5786299999999999E-3</v>
-      </c>
-      <c r="F251">
-        <v>147.46025</v>
-      </c>
-      <c r="G251">
-        <v>147.46025</v>
+        <v>1.43082E-3</v>
+      </c>
+      <c r="F251" s="7">
+        <v>145.03611000000001</v>
+      </c>
+      <c r="G251" s="7">
+        <v>145.03611000000001</v>
       </c>
       <c r="H251">
-        <v>147.46025</v>
+        <v>145.03611000000001</v>
       </c>
       <c r="I251">
-        <v>23.421669999999999</v>
+        <v>14.660428</v>
       </c>
       <c r="J251">
         <v>5</v>
       </c>
-      <c r="K251">
-        <v>147.46025</v>
-      </c>
-      <c r="L251">
-        <v>147.46025</v>
+      <c r="K251" s="7">
+        <v>145.03611000000001</v>
+      </c>
+      <c r="L251" s="2">
+        <v>145.03611000000001</v>
       </c>
       <c r="M251">
-        <v>0.60790999999999995</v>
+        <v>1.7902180000000001</v>
       </c>
       <c r="N251">
         <v>5</v>
       </c>
       <c r="O251" s="2">
-        <v>119.34896000000001</v>
+        <v>115.83778</v>
       </c>
       <c r="P251" s="2">
-        <v>115.65856599999999</v>
+        <v>110.116086</v>
       </c>
       <c r="Q251" t="s">
         <v>367</v>
@@ -16051,7 +16053,7 @@
         <v>392</v>
       </c>
       <c r="B252" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C252">
         <v>7000</v>
@@ -16060,16 +16062,16 @@
         <v>200</v>
       </c>
       <c r="E252" s="1">
-        <v>1.5786299999999999E-3</v>
-      </c>
-      <c r="F252">
-        <v>256.29746</v>
-      </c>
-      <c r="G252">
-        <v>255.91072</v>
+        <v>1.43082E-3</v>
+      </c>
+      <c r="F252" s="7">
+        <v>257.40258999999998</v>
+      </c>
+      <c r="G252" s="7">
+        <v>256.69211000000001</v>
       </c>
       <c r="H252">
-        <v>255.52034399999999</v>
+        <v>255.76541399999999</v>
       </c>
       <c r="I252" t="s">
         <v>367</v>
@@ -16077,23 +16079,23 @@
       <c r="J252">
         <v>0</v>
       </c>
-      <c r="K252">
-        <v>256.29746</v>
-      </c>
-      <c r="L252">
-        <v>256.21625999999998</v>
+      <c r="K252" s="7">
+        <v>257.40258999999998</v>
+      </c>
+      <c r="L252" s="2">
+        <v>257.26673</v>
       </c>
       <c r="M252">
-        <v>41.990220999999998</v>
+        <v>19.674662999999999</v>
       </c>
       <c r="N252">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O252" s="2">
-        <v>198.96678</v>
+        <v>209.70851999999999</v>
       </c>
       <c r="P252" s="2">
-        <v>188.087132</v>
+        <v>198.52690999999999</v>
       </c>
       <c r="Q252" t="s">
         <v>367</v>
@@ -16107,7 +16109,7 @@
         <v>392</v>
       </c>
       <c r="B253" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="C253">
         <v>7000</v>
@@ -16116,16 +16118,16 @@
         <v>300</v>
       </c>
       <c r="E253" s="1">
-        <v>1.5786299999999999E-3</v>
-      </c>
-      <c r="F253">
-        <v>350.39949999999999</v>
-      </c>
-      <c r="G253">
-        <v>349.89794999999998</v>
+        <v>1.43082E-3</v>
+      </c>
+      <c r="F253" s="7">
+        <v>356.18635999999998</v>
+      </c>
+      <c r="G253" s="7">
+        <v>353.43759999999997</v>
       </c>
       <c r="H253">
-        <v>349.11121200000002</v>
+        <v>351.74221199999999</v>
       </c>
       <c r="I253" t="s">
         <v>367</v>
@@ -16133,11 +16135,11 @@
       <c r="J253">
         <v>0</v>
       </c>
-      <c r="K253">
-        <v>350.32562000000001</v>
-      </c>
-      <c r="L253">
-        <v>350.09795600000001</v>
+      <c r="K253" s="7">
+        <v>354.93324000000001</v>
+      </c>
+      <c r="L253" s="2">
+        <v>354.54055199999999</v>
       </c>
       <c r="M253" t="s">
         <v>367</v>
@@ -16146,10 +16148,10 @@
         <v>0</v>
       </c>
       <c r="O253" s="2">
-        <v>267.4271</v>
+        <v>265.5181</v>
       </c>
       <c r="P253" s="2">
-        <v>250.31087199999999</v>
+        <v>262.12535600000001</v>
       </c>
       <c r="Q253" t="s">
         <v>367</v>
@@ -16163,7 +16165,7 @@
         <v>392</v>
       </c>
       <c r="B254" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C254">
         <v>7000</v>
@@ -16172,16 +16174,16 @@
         <v>400</v>
       </c>
       <c r="E254" s="1">
-        <v>1.5786299999999999E-3</v>
-      </c>
-      <c r="F254">
-        <v>435.43218000000002</v>
-      </c>
-      <c r="G254">
-        <v>433.73253</v>
+        <v>1.43082E-3</v>
+      </c>
+      <c r="F254" s="7">
+        <v>447.37688000000003</v>
+      </c>
+      <c r="G254" s="7">
+        <v>444.19513000000001</v>
       </c>
       <c r="H254">
-        <v>432.65671800000001</v>
+        <v>443.39804600000002</v>
       </c>
       <c r="I254" t="s">
         <v>367</v>
@@ -16189,23 +16191,23 @@
       <c r="J254">
         <v>0</v>
       </c>
-      <c r="K254">
-        <v>435.43218000000002</v>
-      </c>
-      <c r="L254">
-        <v>435.06743399999999</v>
-      </c>
-      <c r="M254">
-        <v>28.372845999999999</v>
+      <c r="K254" s="7">
+        <v>446.64213999999998</v>
+      </c>
+      <c r="L254" s="2">
+        <v>446.211344</v>
+      </c>
+      <c r="M254" t="s">
+        <v>367</v>
       </c>
       <c r="N254">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O254" s="2">
-        <v>314.36304000000001</v>
+        <v>328.1669</v>
       </c>
       <c r="P254" s="2">
-        <v>303.00376</v>
+        <v>317.77804600000002</v>
       </c>
       <c r="Q254" t="s">
         <v>367</v>
@@ -16219,7 +16221,7 @@
         <v>392</v>
       </c>
       <c r="B255" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C255">
         <v>7000</v>
@@ -16228,16 +16230,16 @@
         <v>500</v>
       </c>
       <c r="E255" s="1">
-        <v>1.5786299999999999E-3</v>
-      </c>
-      <c r="F255">
-        <v>512.72307999999998</v>
-      </c>
-      <c r="G255">
-        <v>511.16978</v>
+        <v>1.43082E-3</v>
+      </c>
+      <c r="F255" s="7">
+        <v>533.21672000000001</v>
+      </c>
+      <c r="G255" s="7">
+        <v>530.05841999999996</v>
       </c>
       <c r="H255">
-        <v>510.01304199999998</v>
+        <v>529.08722599999999</v>
       </c>
       <c r="I255" t="s">
         <v>367</v>
@@ -16245,11 +16247,11 @@
       <c r="J255">
         <v>0</v>
       </c>
-      <c r="K255">
-        <v>512.27072999999996</v>
-      </c>
-      <c r="L255">
-        <v>511.92844000000002</v>
+      <c r="K255" s="7">
+        <v>532.58043999999995</v>
+      </c>
+      <c r="L255" s="2">
+        <v>532.263868</v>
       </c>
       <c r="M255" t="s">
         <v>367</v>
@@ -16258,10 +16260,10 @@
         <v>0</v>
       </c>
       <c r="O255" s="2">
-        <v>379.13231999999999</v>
+        <v>381.12632000000002</v>
       </c>
       <c r="P255" s="2">
-        <v>356.768214</v>
+        <v>372.77113000000003</v>
       </c>
       <c r="Q255" t="s">
         <v>367</v>
@@ -16275,7 +16277,7 @@
         <v>392</v>
       </c>
       <c r="B256" t="s">
-        <v>306</v>
+        <v>261</v>
       </c>
       <c r="C256">
         <v>7000</v>
@@ -16284,40 +16286,40 @@
         <v>100</v>
       </c>
       <c r="E256" s="1">
-        <v>1.4308599999999999E-3</v>
-      </c>
-      <c r="F256">
-        <v>145.03611000000001</v>
-      </c>
-      <c r="G256">
-        <v>145.03611000000001</v>
+        <v>1.5328200000000001E-3</v>
+      </c>
+      <c r="F256" s="7">
+        <v>142.71664999999999</v>
+      </c>
+      <c r="G256" s="7">
+        <v>142.71664999999999</v>
       </c>
       <c r="H256">
-        <v>145.03163599999999</v>
+        <v>142.00546</v>
       </c>
       <c r="I256">
-        <v>35.157010999999997</v>
+        <v>44.247017</v>
       </c>
       <c r="J256">
-        <v>4</v>
-      </c>
-      <c r="K256">
-        <v>145.03611000000001</v>
-      </c>
-      <c r="L256">
-        <v>145.03611000000001</v>
+        <v>1</v>
+      </c>
+      <c r="K256" s="7">
+        <v>142.71664999999999</v>
+      </c>
+      <c r="L256" s="2">
+        <v>142.71664999999999</v>
       </c>
       <c r="M256">
-        <v>2.1334599999999999</v>
+        <v>1.36968</v>
       </c>
       <c r="N256">
         <v>5</v>
       </c>
       <c r="O256" s="2">
-        <v>115.83778</v>
+        <v>113.59756</v>
       </c>
       <c r="P256" s="2">
-        <v>110.116086</v>
+        <v>109.171176</v>
       </c>
       <c r="Q256" t="s">
         <v>367</v>
@@ -16331,7 +16333,7 @@
         <v>392</v>
       </c>
       <c r="B257" t="s">
-        <v>307</v>
+        <v>262</v>
       </c>
       <c r="C257">
         <v>7000</v>
@@ -16340,16 +16342,16 @@
         <v>200</v>
       </c>
       <c r="E257" s="1">
-        <v>1.4308599999999999E-3</v>
-      </c>
-      <c r="F257">
-        <v>257.40258999999998</v>
-      </c>
-      <c r="G257">
-        <v>256.70634000000001</v>
+        <v>1.5328200000000001E-3</v>
+      </c>
+      <c r="F257" s="7">
+        <v>255.61268999999999</v>
+      </c>
+      <c r="G257" s="7">
+        <v>255.14313999999999</v>
       </c>
       <c r="H257">
-        <v>255.58998600000001</v>
+        <v>254.44111000000001</v>
       </c>
       <c r="I257" t="s">
         <v>367</v>
@@ -16357,23 +16359,23 @@
       <c r="J257">
         <v>0</v>
       </c>
-      <c r="K257">
-        <v>257.40258999999998</v>
-      </c>
-      <c r="L257">
-        <v>257.28757400000001</v>
-      </c>
-      <c r="M257">
-        <v>5.9013400000000003</v>
+      <c r="K257" s="7">
+        <v>255.5487</v>
+      </c>
+      <c r="L257" s="2">
+        <v>255.54099199999999</v>
+      </c>
+      <c r="M257" t="s">
+        <v>367</v>
       </c>
       <c r="N257">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O257" s="2">
-        <v>209.70851999999999</v>
+        <v>200.62246999999999</v>
       </c>
       <c r="P257" s="2">
-        <v>198.52690999999999</v>
+        <v>195.100988</v>
       </c>
       <c r="Q257" t="s">
         <v>367</v>
@@ -16387,7 +16389,7 @@
         <v>392</v>
       </c>
       <c r="B258" t="s">
-        <v>308</v>
+        <v>263</v>
       </c>
       <c r="C258">
         <v>7000</v>
@@ -16396,16 +16398,16 @@
         <v>300</v>
       </c>
       <c r="E258" s="1">
-        <v>1.4308599999999999E-3</v>
-      </c>
-      <c r="F258">
-        <v>356.18635999999998</v>
-      </c>
-      <c r="G258">
-        <v>352.94099999999997</v>
+        <v>1.5328200000000001E-3</v>
+      </c>
+      <c r="F258" s="7">
+        <v>354.48030999999997</v>
+      </c>
+      <c r="G258" s="7">
+        <v>353.61534999999998</v>
       </c>
       <c r="H258">
-        <v>352.20198399999998</v>
+        <v>352.773302</v>
       </c>
       <c r="I258" t="s">
         <v>367</v>
@@ -16413,11 +16415,11 @@
       <c r="J258">
         <v>0</v>
       </c>
-      <c r="K258">
-        <v>354.89026000000001</v>
-      </c>
-      <c r="L258">
-        <v>354.64640600000001</v>
+      <c r="K258" s="7">
+        <v>354.41550000000001</v>
+      </c>
+      <c r="L258" s="2">
+        <v>354.26106199999998</v>
       </c>
       <c r="M258" t="s">
         <v>367</v>
@@ -16426,10 +16428,10 @@
         <v>0</v>
       </c>
       <c r="O258" s="2">
-        <v>265.5181</v>
+        <v>257.99099000000001</v>
       </c>
       <c r="P258" s="2">
-        <v>262.12535600000001</v>
+        <v>247.200424</v>
       </c>
       <c r="Q258" t="s">
         <v>367</v>
@@ -16443,7 +16445,7 @@
         <v>392</v>
       </c>
       <c r="B259" t="s">
-        <v>309</v>
+        <v>264</v>
       </c>
       <c r="C259">
         <v>7000</v>
@@ -16452,16 +16454,16 @@
         <v>400</v>
       </c>
       <c r="E259" s="1">
-        <v>1.4308599999999999E-3</v>
-      </c>
-      <c r="F259">
-        <v>447.37688000000003</v>
-      </c>
-      <c r="G259">
-        <v>444.83702</v>
+        <v>1.5328200000000001E-3</v>
+      </c>
+      <c r="F259" s="7">
+        <v>442.88303999999999</v>
+      </c>
+      <c r="G259" s="7">
+        <v>440.51258999999999</v>
       </c>
       <c r="H259">
-        <v>442.680902</v>
+        <v>439.09607399999999</v>
       </c>
       <c r="I259" t="s">
         <v>367</v>
@@ -16469,11 +16471,11 @@
       <c r="J259">
         <v>0</v>
       </c>
-      <c r="K259">
-        <v>446.34676999999999</v>
-      </c>
-      <c r="L259">
-        <v>446.04652199999998</v>
+      <c r="K259" s="7">
+        <v>442.50301000000002</v>
+      </c>
+      <c r="L259" s="2">
+        <v>442.09483599999999</v>
       </c>
       <c r="M259" t="s">
         <v>367</v>
@@ -16482,10 +16484,10 @@
         <v>0</v>
       </c>
       <c r="O259" s="2">
-        <v>328.1669</v>
+        <v>303.73565000000002</v>
       </c>
       <c r="P259" s="2">
-        <v>317.77804600000002</v>
+        <v>294.27895599999999</v>
       </c>
       <c r="Q259" t="s">
         <v>367</v>
@@ -16499,7 +16501,7 @@
         <v>392</v>
       </c>
       <c r="B260" t="s">
-        <v>310</v>
+        <v>265</v>
       </c>
       <c r="C260">
         <v>7000</v>
@@ -16508,16 +16510,16 @@
         <v>500</v>
       </c>
       <c r="E260" s="1">
-        <v>1.4308599999999999E-3</v>
-      </c>
-      <c r="F260">
-        <v>533.21672000000001</v>
-      </c>
-      <c r="G260">
-        <v>530.67209000000003</v>
+        <v>1.5328200000000001E-3</v>
+      </c>
+      <c r="F260" s="7">
+        <v>524.14255000000003</v>
+      </c>
+      <c r="G260" s="7">
+        <v>521.37064999999996</v>
       </c>
       <c r="H260">
-        <v>529.58963400000005</v>
+        <v>520.72209799999996</v>
       </c>
       <c r="I260" t="s">
         <v>367</v>
@@ -16525,11 +16527,11 @@
       <c r="J260">
         <v>0</v>
       </c>
-      <c r="K260">
-        <v>532.37554</v>
-      </c>
-      <c r="L260">
-        <v>532.15853200000004</v>
+      <c r="K260" s="7">
+        <v>523.64688999999998</v>
+      </c>
+      <c r="L260" s="2">
+        <v>523.14608399999997</v>
       </c>
       <c r="M260" t="s">
         <v>367</v>
@@ -16538,10 +16540,10 @@
         <v>0</v>
       </c>
       <c r="O260" s="2">
-        <v>381.12632000000002</v>
+        <v>375.50416999999999</v>
       </c>
       <c r="P260" s="2">
-        <v>372.77113000000003</v>
+        <v>364.401656</v>
       </c>
       <c r="Q260" t="s">
         <v>367</v>
@@ -16561,39 +16563,39 @@
       <c r="D261" s="8"/>
       <c r="E261" s="9"/>
       <c r="F261" s="8"/>
-      <c r="G261" s="8">
+      <c r="G261" s="12">
         <f t="array" ref="G261">AVERAGE((F211:F260-G211:G260)/F211:F260)</f>
-        <v>2.6214849643415423E-3</v>
-      </c>
-      <c r="H261" s="8">
+        <v>2.6957450207992727E-3</v>
+      </c>
+      <c r="H261" s="12">
         <f t="array" ref="H261">AVERAGE((F211:F260-H211:H260)/F211:F260)</f>
-        <v>4.8701247413402617E-3</v>
+        <v>4.6414921834512816E-3</v>
       </c>
       <c r="I261" s="8"/>
       <c r="J261" s="8">
         <f>SUM(J211:J260)</f>
-        <v>19</v>
-      </c>
-      <c r="K261" s="8">
+        <v>27</v>
+      </c>
+      <c r="K261" s="12">
         <f t="array" ref="K261">AVERAGE((F211:F260-K211:K260)/F211:F260)</f>
-        <v>6.3619381944724342E-4</v>
-      </c>
-      <c r="L261" s="8">
+        <v>5.7301525945369601E-4</v>
+      </c>
+      <c r="L261" s="12">
         <f t="array" ref="L261">AVERAGE((F211:F260-L211:L260)/F211:F260)</f>
-        <v>1.0789381756105482E-3</v>
+        <v>9.6979604099909082E-4</v>
       </c>
       <c r="M261" s="8"/>
       <c r="N261" s="8">
         <f>SUM(N211:N260)</f>
-        <v>72</v>
-      </c>
-      <c r="O261" s="10">
+        <v>77</v>
+      </c>
+      <c r="O261" s="12">
         <f t="array" ref="O261">AVERAGE((F211:F260-O211:O260)/F211:F260)</f>
-        <v>0.2526580074031784</v>
-      </c>
-      <c r="P261" s="10">
+        <v>0.25265676572008156</v>
+      </c>
+      <c r="P261" s="12">
         <f t="array" ref="P261">AVERAGE((F211:F260-P211:P260)/F211:F260)</f>
-        <v>0.28801244013039012</v>
+        <v>0.28795986062188328</v>
       </c>
       <c r="Q261" s="8"/>
       <c r="R261" s="8">
@@ -16747,7 +16749,7 @@
       <c r="K264">
         <v>322.22865999999999</v>
       </c>
-      <c r="L264">
+      <c r="L264" s="16">
         <v>321.97440599999999</v>
       </c>
       <c r="M264" t="s">
@@ -16791,8 +16793,8 @@
       <c r="G265">
         <v>392.06358999999998</v>
       </c>
-      <c r="H265">
-        <v>390.24020400000001</v>
+      <c r="H265" s="16">
+        <v>390.38539200000002</v>
       </c>
       <c r="I265" t="s">
         <v>367</v>
@@ -16803,8 +16805,8 @@
       <c r="K265">
         <v>393.96911</v>
       </c>
-      <c r="L265">
-        <v>393.54638999999997</v>
+      <c r="L265" s="16">
+        <v>393.52470799999998</v>
       </c>
       <c r="M265" t="s">
         <v>367</v>
@@ -16812,11 +16814,11 @@
       <c r="N265">
         <v>0</v>
       </c>
-      <c r="O265" s="7">
+      <c r="O265" s="19">
         <v>290.55641000000003</v>
       </c>
-      <c r="P265" s="2">
-        <v>268.12577800000003</v>
+      <c r="P265" s="18">
+        <v>261.67109399999998</v>
       </c>
       <c r="Q265" t="s">
         <v>367</v>
@@ -16892,39 +16894,39 @@
       <c r="D267" s="8"/>
       <c r="E267" s="9"/>
       <c r="F267" s="8"/>
-      <c r="G267" s="8">
+      <c r="G267" s="12">
         <f t="array" ref="G267">AVERAGE((F262:F266-G262:G266)/F262:F266)</f>
         <v>8.2269103605319936E-3</v>
       </c>
-      <c r="H267" s="8">
+      <c r="H267" s="12">
         <f t="array" ref="H267">AVERAGE((F262:F266-H262:H266)/F262:F266)</f>
-        <v>1.1735767919018673E-2</v>
+        <v>1.1662644494456319E-2</v>
       </c>
       <c r="I267" s="8"/>
       <c r="J267" s="8">
         <f>SUM(J262:J266)</f>
         <v>0</v>
       </c>
-      <c r="K267" s="8">
+      <c r="K267" s="12">
         <f t="array" ref="K267">AVERAGE((F262:F266-K262:K266)/F262:F266)</f>
         <v>4.0773277962307302E-3</v>
       </c>
-      <c r="L267" s="8">
+      <c r="L267" s="12">
         <f t="array" ref="L267">AVERAGE((F262:F266-L262:L266)/F262:F266)</f>
-        <v>4.7196465190507729E-3</v>
+        <v>4.7305665819441295E-3</v>
       </c>
       <c r="M267" s="8"/>
       <c r="N267" s="8">
         <f>SUM(N262:N266)</f>
         <v>0</v>
       </c>
-      <c r="O267" s="10">
+      <c r="O267" s="12">
         <f t="array" ref="O267">AVERAGE((F262:F266-O262:O266)/F262:F266)</f>
         <v>0.31017737032213855</v>
       </c>
-      <c r="P267" s="10">
+      <c r="P267" s="12">
         <f t="array" ref="P267">AVERAGE((F262:F266-P262:P266)/F262:F266)</f>
-        <v>0.34303704753430464</v>
+        <v>0.34628792638481415</v>
       </c>
       <c r="Q267" s="8"/>
       <c r="R267" s="8">
@@ -19410,11 +19412,11 @@
       <c r="D313" s="8"/>
       <c r="E313" s="9"/>
       <c r="F313" s="8"/>
-      <c r="G313" s="8">
+      <c r="G313" s="17">
         <f t="array" ref="G313">AVERAGE((F276:F312-G276:G312)/F276:F312)</f>
         <v>2.4267485684229956E-3</v>
       </c>
-      <c r="H313" s="8">
+      <c r="H313" s="17">
         <f t="array" ref="H313">AVERAGE((F276:F312-H276:H312)/F276:F312)</f>
         <v>2.5739789420904085E-3</v>
       </c>
@@ -19423,11 +19425,11 @@
         <f>SUM(J276:J312)</f>
         <v>135</v>
       </c>
-      <c r="K313" s="8">
+      <c r="K313" s="17">
         <f t="array" ref="K313">AVERAGE((F276:F312-K276:K312)/F276:F312)</f>
         <v>2.2448027740352059E-3</v>
       </c>
-      <c r="L313" s="8">
+      <c r="L313" s="17">
         <f t="array" ref="L313">AVERAGE((F276:F312-L276:L312)/F276:F312)</f>
         <v>2.3605553781793618E-3</v>
       </c>
@@ -19436,11 +19438,11 @@
         <f>SUM(N276:N312)</f>
         <v>142</v>
       </c>
-      <c r="O313" s="10">
+      <c r="O313" s="17">
         <f t="array" ref="O313">AVERAGE((F276:F312-O276:O312)/F276:F312)</f>
         <v>2.5001749433333355E-3</v>
       </c>
-      <c r="P313" s="10">
+      <c r="P313" s="17">
         <f t="array" ref="P313">AVERAGE((F276:F312-P276:P312)/F276:F312)</f>
         <v>2.7633878534528387E-3</v>
       </c>
@@ -21755,11 +21757,11 @@
       <c r="D355" s="8"/>
       <c r="E355" s="9"/>
       <c r="F355" s="8"/>
-      <c r="G355" s="8">
+      <c r="G355" s="17">
         <f t="array" ref="G355">AVERAGE((F314:F354-G314:G354)/F314:F354)</f>
         <v>5.293460713895517E-4</v>
       </c>
-      <c r="H355" s="8">
+      <c r="H355" s="17">
         <f t="array" ref="H355">AVERAGE((F314:F354-H314:H354)/F314:F354)</f>
         <v>8.6166575562223987E-4</v>
       </c>
@@ -21768,11 +21770,11 @@
         <f>SUM(J314:J354)</f>
         <v>68</v>
       </c>
-      <c r="K355" s="8">
+      <c r="K355" s="17">
         <f t="array" ref="K355">AVERAGE((F314:F354-K314:K354)/F314:F354)</f>
         <v>2.0132481772161531E-4</v>
       </c>
-      <c r="L355" s="8">
+      <c r="L355" s="17">
         <f t="array" ref="L355">AVERAGE((F314:F354-L314:L354)/F314:F354)</f>
         <v>4.3650180524949154E-4</v>
       </c>
@@ -21781,11 +21783,11 @@
         <f>SUM(N314:N354)</f>
         <v>111</v>
       </c>
-      <c r="O355" s="10">
+      <c r="O355" s="17">
         <f t="array" ref="O355">AVERAGE((F314:F354-O314:O354)/F314:F354)</f>
         <v>1.1826429680795736E-3</v>
       </c>
-      <c r="P355" s="10">
+      <c r="P355" s="17">
         <f t="array" ref="P355">AVERAGE((F314:F354-P314:P354)/F314:F354)</f>
         <v>1.648301477585325E-3</v>
       </c>
@@ -22035,10 +22037,10 @@
         <v>130</v>
       </c>
       <c r="G361">
-        <v>148</v>
+        <v>422</v>
       </c>
       <c r="H361">
-        <v>260.60000000000002</v>
+        <v>565.20000000000005</v>
       </c>
       <c r="I361" t="s">
         <v>367</v>
@@ -22050,13 +22052,13 @@
         <v>130</v>
       </c>
       <c r="L361">
-        <v>153.80000000000001</v>
+        <v>130</v>
       </c>
       <c r="M361" s="5">
-        <v>11.322127</v>
+        <v>19.501142000000002</v>
       </c>
       <c r="N361">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="362" spans="1:18" x14ac:dyDescent="0.3">

</xml_diff>